<commit_message>
fix(journal): institutional dynamic Excel formulas across all 3 sheets, isolate realized PnL from open trades, strict closed-only tax compliance
</commit_message>
<xml_diff>
--- a/SkonVault_Live_Transaction_Journal.xlsx
+++ b/SkonVault_Live_Transaction_Journal.xlsx
@@ -11,10 +11,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="&quot;฿&quot;#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="#,##0"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -116,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -140,6 +141,15 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
 </styleSheet>
 </file>
@@ -174,7 +184,7 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
         <is>
-          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-09-29 17:39 ICT</t>
+          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-09-29 22:18 ICT</t>
         </is>
       </c>
     </row>
@@ -186,12 +196,12 @@
       </c>
       <c r="C4" t="inlineStr" s="3">
         <is>
-          <t>Cash Gap to Goal</t>
+          <t>35% Safe Cash Floor</t>
         </is>
       </c>
       <c r="E4" t="inlineStr" s="3">
         <is>
-          <t>Net Cash Injected</t>
+          <t>Active Premium Injected</t>
         </is>
       </c>
       <c r="G4" t="inlineStr" s="3">
@@ -206,29 +216,32 @@
       </c>
       <c r="K4" t="inlineStr" s="3">
         <is>
-          <t>Graduation Status</t>
+          <t>Cash Reserve Health</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6">
-        <v>2135.24</v>
+        <v>32729.7</v>
       </c>
       <c r="C5" s="6">
-        <v>15907.13</v>
+        <v>11249.0</v>
       </c>
       <c r="E5" s="7">
-        <v>150.0</v>
+        <f>J12</f>
+        <v>710.0</v>
       </c>
       <c r="G5" s="7">
-        <v>75.0</v>
+        <f>K12</f>
+        <v>355.0</v>
       </c>
       <c r="I5" s="6">
-        <v>500.0</v>
+        <f>L12</f>
+        <v>4200.0</v>
       </c>
       <c r="K5" t="inlineStr" s="10">
         <is>
-          <t>11.8% ON TRACK (Gap: $15,907.13) 🚀</t>
+          <t>102.3% CASH RESERVE (≥35% FLOOR) 🟢</t>
         </is>
       </c>
     </row>
@@ -317,93 +330,296 @@
       </c>
       <c r="B8" t="inlineStr" s="10">
         <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (#290523608)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="10">
+        <is>
+          <t>$220.00P / $215.00P</t>
+        </is>
+      </c>
+      <c r="E8" s="0">
+        <v>6</v>
+      </c>
+      <c r="F8" s="6">
+        <v>230.54</v>
+      </c>
+      <c r="G8" t="inlineStr" s="7">
+        <is>
+          <t>+$10.54 (+4.6%) OTM Buffer 🟢</t>
+        </is>
+      </c>
+      <c r="H8" s="6">
+        <v>1026.0</v>
+      </c>
+      <c r="I8" s="6">
+        <v>600.0</v>
+      </c>
+      <c r="J8" s="7">
+        <f>H8-I8</f>
+        <v>426.0</v>
+      </c>
+      <c r="K8" s="7">
+        <f>J8*0.5</f>
+        <v>213.0</v>
+      </c>
+      <c r="L8" s="6">
+        <v>3000.0</v>
+      </c>
+      <c r="M8" t="inlineStr" s="0">
+        <is>
+          <t>Oct 07, 2026 (T-3 DTE)</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr" s="0">
+        <is>
+          <t>Oct 12, 2026</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr" s="7">
+        <is>
+          <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="0">
+        <is>
+          <t>3. Inflation Defense &amp; Hard Assets</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="10">
+        <is>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (#290523608)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="10">
+        <is>
+          <t>$60.00P / $58.00P</t>
+        </is>
+      </c>
+      <c r="E9" s="0">
+        <v>1</v>
+      </c>
+      <c r="F9" s="6">
+        <v>61.615</v>
+      </c>
+      <c r="G9" t="inlineStr" s="7">
+        <is>
+          <t>+$1.62 (+2.6%) OTM Buffer 🟢</t>
+        </is>
+      </c>
+      <c r="H9" s="6">
+        <v>68.0</v>
+      </c>
+      <c r="I9" s="6">
+        <v>32.0</v>
+      </c>
+      <c r="J9" s="7">
+        <f>H9-I9</f>
+        <v>36.0</v>
+      </c>
+      <c r="K9" s="7">
+        <f>J9*0.5</f>
+        <v>18.0</v>
+      </c>
+      <c r="L9" s="6">
+        <v>200.0</v>
+      </c>
+      <c r="M9" t="inlineStr" s="0">
+        <is>
+          <t>Oct 13, 2026 (T-3 DTE)</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr" s="0">
+        <is>
+          <t>Oct 16, 2026</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr" s="7">
+        <is>
+          <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="0">
+        <is>
+          <t>8. Mega-Cap Cloud &amp; Software Platform</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="10">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="0">
+        <is>
+          <t>Tradier Live (#6YB80974)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="10">
+        <is>
+          <t>$685.00P / $680.00P</t>
+        </is>
+      </c>
+      <c r="E10" s="0">
+        <v>1</v>
+      </c>
+      <c r="F10" s="6">
+        <v>721.62</v>
+      </c>
+      <c r="G10" t="inlineStr" s="7">
+        <is>
+          <t>+$36.62 (+5.1%) OTM Buffer 🟢</t>
+        </is>
+      </c>
+      <c r="H10" s="6">
+        <v>555.0</v>
+      </c>
+      <c r="I10" s="6">
+        <v>457.0</v>
+      </c>
+      <c r="J10" s="7">
+        <f>H10-I10</f>
+        <v>98.0</v>
+      </c>
+      <c r="K10" s="7">
+        <f>J10*0.5</f>
+        <v>49.0</v>
+      </c>
+      <c r="L10" s="6">
+        <v>500.0</v>
+      </c>
+      <c r="M10" t="inlineStr" s="0">
+        <is>
+          <t>Oct 06, 2026 (T-3 DTE)</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr" s="0">
+        <is>
+          <t>Oct 09, 2026</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr" s="7">
+        <is>
+          <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="0">
+        <is>
+          <t>1. AI Chips &amp; Hardware</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="10">
+        <is>
           <t>TSM</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr" s="0">
+      <c r="C11" t="inlineStr" s="0">
         <is>
           <t>Tradier Live (#6YB80974)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr" s="10">
+      <c r="D11" t="inlineStr" s="10">
         <is>
           <t>$425.00P / $420.00P</t>
         </is>
       </c>
-      <c r="E8" s="0">
+      <c r="E11" s="0">
         <v>1</v>
       </c>
-      <c r="F8" s="6">
-        <v>452.88</v>
-      </c>
-      <c r="G8" t="inlineStr" s="7">
-        <is>
-          <t>+$27.88 (+6.2%) OTM Buffer 🟢</t>
-        </is>
-      </c>
-      <c r="H8" s="6">
+      <c r="F11" s="6">
+        <v>455.62</v>
+      </c>
+      <c r="G11" t="inlineStr" s="7">
+        <is>
+          <t>+$30.62 (+6.7%) OTM Buffer 🟢</t>
+        </is>
+      </c>
+      <c r="H11" s="6">
         <v>897.0</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I11" s="6">
         <v>747.0</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J11" s="7">
+        <f>H11-I11</f>
         <v>150.0</v>
       </c>
-      <c r="K8" s="7">
+      <c r="K11" s="7">
+        <f>J11*0.5</f>
         <v>75.0</v>
       </c>
-      <c r="L8" s="6">
+      <c r="L11" s="6">
         <v>500.0</v>
       </c>
-      <c r="M8" t="inlineStr" s="0">
+      <c r="M11" t="inlineStr" s="0">
         <is>
           <t>Oct 27, 2026 (T-3 DTE)</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr" s="0">
+      <c r="N11" t="inlineStr" s="0">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr" s="7">
+      <c r="O11" t="inlineStr" s="7">
         <is>
           <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr" s="5">
+    <row r="12">
+      <c r="A12" t="inlineStr" s="5">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5">
-        <v>1</v>
-      </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5">
-        <v>897.0</v>
-      </c>
-      <c r="I9" s="5">
-        <v>747.0</v>
-      </c>
-      <c r="J9" s="5">
-        <v>150.0</v>
-      </c>
-      <c r="K9" s="5">
-        <v>75.0</v>
-      </c>
-      <c r="L9" s="5">
-        <v>500.0</v>
-      </c>
-      <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" t="inlineStr" s="5">
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="13">
+        <f>SUM(E8:E11)</f>
+        <v>9</v>
+      </c>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="11">
+        <f>SUM(H8:H11)</f>
+        <v>2546.0</v>
+      </c>
+      <c r="I12" s="11">
+        <f>SUM(I8:I11)</f>
+        <v>1836.0</v>
+      </c>
+      <c r="J12" s="11">
+        <f>SUM(J8:J11)</f>
+        <v>710.0</v>
+      </c>
+      <c r="K12" s="11">
+        <f>SUM(K8:K11)</f>
+        <v>355.0</v>
+      </c>
+      <c r="L12" s="11">
+        <f>SUM(L8:L11)</f>
+        <v>4200.0</v>
+      </c>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
+      <c r="O12" t="inlineStr" s="5">
         <is>
           <t>100% DEFINED RISK PROTECTED ✅</t>
         </is>
@@ -445,7 +661,7 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
         <is>
-          <t>Historical Execution Log — Reconciled with Alpaca REST API</t>
+          <t>Historical Execution Log — Reconciled with Live Broker REST APIs (Alpaca &amp; Tradier)</t>
         </is>
       </c>
     </row>
@@ -577,9 +793,720 @@
       </c>
       <c r="Z4" t="inlineStr" s="3">
         <is>
-          <t>Alpaca Order ID</t>
-        </is>
-      </c>
+          <t>Broker Order ID</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="0">
+        <is>
+          <t>TRD-20260908-XLF-54/52</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (#290523608)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="10">
+        <is>
+          <t>XLF</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="0">
+        <is>
+          <t>6. Financial Services &amp; Payment Rails</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="0">
+        <is>
+          <t>Bull Put Spread (54P/52P)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr" s="0">
+        <is>
+          <t>15:09:30</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr" s="0">
+        <is>
+          <t>XLF261016P00054000</t>
+        </is>
+      </c>
+      <c r="I5" s="6">
+        <v>54.0</v>
+      </c>
+      <c r="J5" t="inlineStr" s="0">
+        <is>
+          <t>XLF261016P00052000</t>
+        </is>
+      </c>
+      <c r="K5" s="6">
+        <v>52.0</v>
+      </c>
+      <c r="L5" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="M5" s="0">
+        <v>1</v>
+      </c>
+      <c r="N5" s="6">
+        <v>0.11</v>
+      </c>
+      <c r="O5" s="6">
+        <v>11.0</v>
+      </c>
+      <c r="P5" s="6">
+        <v>200.0</v>
+      </c>
+      <c r="Q5" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr" s="0">
+        <is>
+          <t>13:36:45</t>
+        </is>
+      </c>
+      <c r="S5" s="6">
+        <v>0.44</v>
+      </c>
+      <c r="T5" s="6">
+        <v>44.0</v>
+      </c>
+      <c r="U5" s="6">
+        <f>O5-T5</f>
+        <v>-33.0</v>
+      </c>
+      <c r="V5" s="8">
+        <f>IF(P5&gt;0,U5/P5,0)</f>
+        <v>-0.165</v>
+      </c>
+      <c r="W5" s="0">
+        <v>406.5</v>
+      </c>
+      <c r="X5" t="inlineStr" s="0">
+        <is>
+          <t>Defensive stop-out / loss close (verified fill)</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr" s="10">
+        <is>
+          <t>CLOSED_DEFENSIVE</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr" s="0">
+        <is>
+          <t>754fde1f-10f6-44f0-afc9-4d6b8f0ba882</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="0">
+        <is>
+          <t>TRD-20260908-XLF-54/53</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="0">
+        <is>
+          <t>Tradier Live (#6YB80974)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="10">
+        <is>
+          <t>XLF</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="0">
+        <is>
+          <t>6. Financial Services &amp; Payment Rails</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="0">
+        <is>
+          <t>Bull Put Spread (54P/53P)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr" s="0">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr" s="0">
+        <is>
+          <t>XLF261016P00054000</t>
+        </is>
+      </c>
+      <c r="I6" s="6">
+        <v>54.0</v>
+      </c>
+      <c r="J6" t="inlineStr" s="0">
+        <is>
+          <t>XLF261016P00053000</t>
+        </is>
+      </c>
+      <c r="K6" s="6">
+        <v>53.0</v>
+      </c>
+      <c r="L6" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="M6" s="0">
+        <v>1</v>
+      </c>
+      <c r="N6" s="6">
+        <v>0.08</v>
+      </c>
+      <c r="O6" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="P6" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="Q6" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr" s="0">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+      <c r="S6" s="6">
+        <v>0.35</v>
+      </c>
+      <c r="T6" s="6">
+        <v>35.0</v>
+      </c>
+      <c r="U6" s="6">
+        <f>O6-T6</f>
+        <v>-27.0</v>
+      </c>
+      <c r="V6" s="8">
+        <f>IF(P6&gt;0,U6/P6,0)</f>
+        <v>-0.27</v>
+      </c>
+      <c r="W6" s="0">
+        <v>480.0</v>
+      </c>
+      <c r="X6" t="inlineStr" s="0">
+        <is>
+          <t>Defensive stop-out / loss close (verified fill)</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr" s="10">
+        <is>
+          <t>CLOSED_DEFENSIVE</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr" s="0">
+        <is>
+          <t>tradier_2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="0">
+        <is>
+          <t>TRD-20260921-XLE-60/58</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (#290523608)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="10">
+        <is>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="0">
+        <is>
+          <t>3. Inflation Defense &amp; Hard Assets</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="0">
+        <is>
+          <t>Bull Put Spread (60P/58P)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr" s="0">
+        <is>
+          <t>19:21:19</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr" s="0">
+        <is>
+          <t>XLE261016P00060000</t>
+        </is>
+      </c>
+      <c r="I7" s="6">
+        <v>60.0</v>
+      </c>
+      <c r="J7" t="inlineStr" s="0">
+        <is>
+          <t>XLE261016P00058000</t>
+        </is>
+      </c>
+      <c r="K7" s="6">
+        <v>58.0</v>
+      </c>
+      <c r="L7" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="M7" s="0">
+        <v>1</v>
+      </c>
+      <c r="N7" s="6">
+        <v>0.36</v>
+      </c>
+      <c r="O7" s="6">
+        <v>36.0</v>
+      </c>
+      <c r="P7" s="6">
+        <v>200.0</v>
+      </c>
+      <c r="Q7" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S7" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="T7" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="U7" s="6">
+        <v>0.00</v>
+      </c>
+      <c r="V7" s="8">
+        <v>0.0</v>
+      </c>
+      <c r="W7" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="X7" t="inlineStr" s="0">
+        <is>
+          <t>Active with broker (live position)</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr" s="10">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr" s="0">
+        <is>
+          <t>e581bd48-ad5a-4ea2-b0b3-db33118a637b</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="0">
+        <is>
+          <t>TRD-20260928-NVDA-220/215</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (#290523608)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="10">
+        <is>
+          <t>NVDA</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="0">
+        <is>
+          <t>1. AI Chips &amp; Hardware</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="0">
+        <is>
+          <t>Bull Put Spread (220P/215P)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr" s="0">
+        <is>
+          <t>14:16:24</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr" s="0">
+        <is>
+          <t>NVDA261012P00220000</t>
+        </is>
+      </c>
+      <c r="I8" s="6">
+        <v>220.0</v>
+      </c>
+      <c r="J8" t="inlineStr" s="0">
+        <is>
+          <t>NVDA261012P00215000</t>
+        </is>
+      </c>
+      <c r="K8" s="6">
+        <v>215.0</v>
+      </c>
+      <c r="L8" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="M8" s="0">
+        <v>6</v>
+      </c>
+      <c r="N8" s="6">
+        <v>0.71</v>
+      </c>
+      <c r="O8" s="6">
+        <v>426.0</v>
+      </c>
+      <c r="P8" s="6">
+        <v>3000.0</v>
+      </c>
+      <c r="Q8" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S8" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="T8" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="U8" s="6">
+        <v>0.00</v>
+      </c>
+      <c r="V8" s="8">
+        <v>0.0</v>
+      </c>
+      <c r="W8" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="X8" t="inlineStr" s="0">
+        <is>
+          <t>Active with broker (live position)</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr" s="10">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr" s="0">
+        <is>
+          <t>b62cee06-2bd9-43c4-a8ce-53385fad4b19</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="0">
+        <is>
+          <t>TRD-20260928-TSM-425/420</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="0">
+        <is>
+          <t>Tradier Live (#6YB80974)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="10">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="0">
+        <is>
+          <t>1. AI Chips &amp; Hardware</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="0">
+        <is>
+          <t>Bull Put Spread (425P/420P)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr" s="0">
+        <is>
+          <t>00:00:00</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr" s="0">
+        <is>
+          <t>TSM261030P00425000</t>
+        </is>
+      </c>
+      <c r="I9" s="6">
+        <v>425.0</v>
+      </c>
+      <c r="J9" t="inlineStr" s="0">
+        <is>
+          <t>TSM261030P00420000</t>
+        </is>
+      </c>
+      <c r="K9" s="6">
+        <v>420.0</v>
+      </c>
+      <c r="L9" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="M9" s="0">
+        <v>1</v>
+      </c>
+      <c r="N9" s="6">
+        <v>1.5</v>
+      </c>
+      <c r="O9" s="6">
+        <v>150.0</v>
+      </c>
+      <c r="P9" s="6">
+        <v>500.0</v>
+      </c>
+      <c r="Q9" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S9" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="T9" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="U9" s="6">
+        <v>0.00</v>
+      </c>
+      <c r="V9" s="8">
+        <v>0.0</v>
+      </c>
+      <c r="W9" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="X9" t="inlineStr" s="0">
+        <is>
+          <t>Active with broker (live position)</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr" s="10">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr" s="0">
+        <is>
+          <t>tradier_2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="0">
+        <is>
+          <t>TRD-20260929-META-685/680</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="0">
+        <is>
+          <t>Tradier Live (#6YB80974)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="10">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="0">
+        <is>
+          <t>8. Mega-Cap Cloud &amp; Software Platform</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="0">
+        <is>
+          <t>Bull Put Spread (685P/680P)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr" s="0">
+        <is>
+          <t>14:16:18</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr" s="0">
+        <is>
+          <t>META261009P00685000</t>
+        </is>
+      </c>
+      <c r="I10" s="6">
+        <v>685.0</v>
+      </c>
+      <c r="J10" t="inlineStr" s="0">
+        <is>
+          <t>META261009P00680000</t>
+        </is>
+      </c>
+      <c r="K10" s="6">
+        <v>680.0</v>
+      </c>
+      <c r="L10" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M10" s="0">
+        <v>1</v>
+      </c>
+      <c r="N10" s="6">
+        <v>0.98</v>
+      </c>
+      <c r="O10" s="6">
+        <v>98.0</v>
+      </c>
+      <c r="P10" s="6">
+        <v>500.0</v>
+      </c>
+      <c r="Q10" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S10" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="T10" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="U10" s="6">
+        <v>0.00</v>
+      </c>
+      <c r="V10" s="8">
+        <v>0.0</v>
+      </c>
+      <c r="W10" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="X10" t="inlineStr" s="0">
+        <is>
+          <t>Active with broker (live position)</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr" s="10">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr" s="0">
+        <is>
+          <t>148305471</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="5">
+        <is>
+          <t>TOTALS / RECONCILED</t>
+        </is>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="13">
+        <f>SUM(M5:M10)</f>
+        <v>11</v>
+      </c>
+      <c r="N11" s="5"/>
+      <c r="O11" s="11">
+        <f>SUM(O5:O10)</f>
+        <v>729.0</v>
+      </c>
+      <c r="P11" s="11">
+        <f>SUM(P5:P10)</f>
+        <v>4500.0</v>
+      </c>
+      <c r="Q11" s="5"/>
+      <c r="R11" s="5"/>
+      <c r="S11" s="5"/>
+      <c r="T11" s="11">
+        <f>SUM(T5:T10)</f>
+        <v>79.0</v>
+      </c>
+      <c r="U11" s="11">
+        <f>SUM(U5:U10)</f>
+        <v>-60.0</v>
+      </c>
+      <c r="V11" s="5"/>
+      <c r="W11" s="5"/>
+      <c r="X11" s="5"/>
+      <c r="Y11" s="5"/>
+      <c r="Z11" s="5"/>
     </row>
   </sheetData>
 </worksheet>
@@ -676,6 +1603,149 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="0">
+        <is>
+          <t>TAX-20260908-XLF-54/52</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Securities LLC</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="0">
+        <is>
+          <t>290523608</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="10">
+        <is>
+          <t>XLF</t>
+        </is>
+      </c>
+      <c r="F5" s="6">
+        <v>11.0</v>
+      </c>
+      <c r="G5" s="6">
+        <v>44.0</v>
+      </c>
+      <c r="H5" s="6">
+        <f>F5-G5</f>
+        <v>-33.0</v>
+      </c>
+      <c r="I5" s="6">
+        <v>36.5</v>
+      </c>
+      <c r="J5" s="9">
+        <f>IF(H5&gt;0,H5*I5,0)</f>
+        <v>0.0</v>
+      </c>
+      <c r="K5" s="9">
+        <f>J5</f>
+        <v>0.0</v>
+      </c>
+      <c r="L5" t="inlineStr" s="0">
+        <is>
+          <t>754fde1f-10f6-44f0-afc9-4d6b8f0ba882</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="0">
+        <is>
+          <t>TAX-20260908-XLF-54/53</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="0">
+        <is>
+          <t>Tradier (Apex Clearing Corp)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="0">
+        <is>
+          <t>6YB80974</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="10">
+        <is>
+          <t>XLF</t>
+        </is>
+      </c>
+      <c r="F6" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="G6" s="6">
+        <v>35.0</v>
+      </c>
+      <c r="H6" s="6">
+        <f>F6-G6</f>
+        <v>-27.0</v>
+      </c>
+      <c r="I6" s="6">
+        <v>36.5</v>
+      </c>
+      <c r="J6" s="9">
+        <f>IF(H6&gt;0,H6*I6,0)</f>
+        <v>0.0</v>
+      </c>
+      <c r="K6" s="9">
+        <f>J6</f>
+        <v>0.0</v>
+      </c>
+      <c r="L6" t="inlineStr" s="0">
+        <is>
+          <t>tradier_2026-09-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="5">
+        <is>
+          <t>TOTAL CLOSED REVENUE</t>
+        </is>
+      </c>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="11">
+        <f>SUM(F5:F6)</f>
+        <v>19.0</v>
+      </c>
+      <c r="G7" s="11">
+        <f>SUM(G5:G6)</f>
+        <v>79.0</v>
+      </c>
+      <c r="H7" s="11">
+        <f>SUM(H5:H6)</f>
+        <v>-60.0</v>
+      </c>
+      <c r="I7" s="5"/>
+      <c r="J7" s="12">
+        <f>SUM(J5:J6)</f>
+        <v>0.0</v>
+      </c>
+      <c r="K7" s="12">
+        <f>SUM(K5:K6)</f>
+        <v>0.0</v>
+      </c>
+      <c r="L7" t="inlineStr" s="5">
+        <is>
+          <t>AUDITED COMPLIANT ✅</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore(sync): nightly live transaction journals and runtime states (2026-09-30)
</commit_message>
<xml_diff>
--- a/SkonVault_Live_Transaction_Journal.xlsx
+++ b/SkonVault_Live_Transaction_Journal.xlsx
@@ -184,7 +184,7 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
         <is>
-          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-09-29 22:18 ICT</t>
+          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-09-30 22:53 ICT</t>
         </is>
       </c>
     </row>
@@ -222,26 +222,26 @@
     </row>
     <row r="5">
       <c r="A5" s="6">
-        <v>32729.7</v>
+        <v>34634.77</v>
       </c>
       <c r="C5" s="6">
         <v>11249.0</v>
       </c>
       <c r="E5" s="7">
-        <f>J12</f>
-        <v>710.0</v>
+        <f>J15</f>
+        <v>2616.0</v>
       </c>
       <c r="G5" s="7">
-        <f>K12</f>
-        <v>355.0</v>
+        <f>K15</f>
+        <v>1308.0</v>
       </c>
       <c r="I5" s="6">
-        <f>L12</f>
-        <v>4200.0</v>
+        <f>L15</f>
+        <v>21200.0</v>
       </c>
       <c r="K5" t="inlineStr" s="10">
         <is>
-          <t>102.3% CASH RESERVE (≥35% FLOOR) 🟢</t>
+          <t>108.2% CASH RESERVE (≥35% FLOOR) 🟢</t>
         </is>
       </c>
     </row>
@@ -330,7 +330,7 @@
       </c>
       <c r="B8" t="inlineStr" s="10">
         <is>
-          <t>NVDA</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="0">
@@ -340,45 +340,45 @@
       </c>
       <c r="D8" t="inlineStr" s="10">
         <is>
-          <t>$220.00P / $215.00P</t>
+          <t>$335.00P / $305.00P</t>
         </is>
       </c>
       <c r="E8" s="0">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F8" s="6">
-        <v>230.54</v>
+        <v>354.2875</v>
       </c>
       <c r="G8" t="inlineStr" s="7">
         <is>
-          <t>+$10.54 (+4.6%) OTM Buffer 🟢</t>
+          <t>+$19.29 (+5.4%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H8" s="6">
-        <v>1026.0</v>
+        <v>978.0</v>
       </c>
       <c r="I8" s="6">
-        <v>600.0</v>
+        <v>111.0</v>
       </c>
       <c r="J8" s="7">
         <f>H8-I8</f>
-        <v>426.0</v>
+        <v>867.0</v>
       </c>
       <c r="K8" s="7">
         <f>J8*0.5</f>
-        <v>213.0</v>
+        <v>433.5</v>
       </c>
       <c r="L8" s="6">
-        <v>3000.0</v>
+        <v>9000.0</v>
       </c>
       <c r="M8" t="inlineStr" s="0">
         <is>
-          <t>Oct 07, 2026 (T-3 DTE)</t>
+          <t>Oct 13, 2026 (T-3 DTE)</t>
         </is>
       </c>
       <c r="N8" t="inlineStr" s="0">
         <is>
-          <t>Oct 12, 2026</t>
+          <t>Oct 16, 2026</t>
         </is>
       </c>
       <c r="O8" t="inlineStr" s="7">
@@ -390,12 +390,12 @@
     <row r="9">
       <c r="A9" t="inlineStr" s="0">
         <is>
-          <t>3. Inflation Defense &amp; Hard Assets</t>
+          <t>1. AI Chips &amp; Hardware</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="10">
         <is>
-          <t>XLE</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="0">
@@ -405,45 +405,45 @@
       </c>
       <c r="D9" t="inlineStr" s="10">
         <is>
-          <t>$60.00P / $58.00P</t>
+          <t>$220.00P / $215.00P</t>
         </is>
       </c>
       <c r="E9" s="0">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F9" s="6">
-        <v>61.615</v>
+        <v>231.05</v>
       </c>
       <c r="G9" t="inlineStr" s="7">
         <is>
-          <t>+$1.62 (+2.6%) OTM Buffer 🟢</t>
+          <t>+$11.05 (+4.8%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H9" s="6">
-        <v>68.0</v>
+        <v>1026.0</v>
       </c>
       <c r="I9" s="6">
-        <v>32.0</v>
+        <v>600.0</v>
       </c>
       <c r="J9" s="7">
         <f>H9-I9</f>
-        <v>36.0</v>
+        <v>426.0</v>
       </c>
       <c r="K9" s="7">
         <f>J9*0.5</f>
-        <v>18.0</v>
+        <v>213.0</v>
       </c>
       <c r="L9" s="6">
-        <v>200.0</v>
+        <v>3000.0</v>
       </c>
       <c r="M9" t="inlineStr" s="0">
         <is>
-          <t>Oct 13, 2026 (T-3 DTE)</t>
+          <t>Oct 07, 2026 (T-3 DTE)</t>
         </is>
       </c>
       <c r="N9" t="inlineStr" s="0">
         <is>
-          <t>Oct 16, 2026</t>
+          <t>Oct 12, 2026</t>
         </is>
       </c>
       <c r="O9" t="inlineStr" s="7">
@@ -455,60 +455,60 @@
     <row r="10">
       <c r="A10" t="inlineStr" s="0">
         <is>
-          <t>8. Mega-Cap Cloud &amp; Software Platform</t>
+          <t>7. Broad Index &amp; Market Hedging</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="10">
         <is>
-          <t>META</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="0">
         <is>
-          <t>Tradier Live (#6YB80974)</t>
+          <t>Alpaca Live (#290523608)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="10">
         <is>
-          <t>$685.00P / $680.00P</t>
+          <t>$700P/$675P &amp; $775C/$800C (IC)</t>
         </is>
       </c>
       <c r="E10" s="0">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" s="6">
-        <v>721.62</v>
+        <v>745.05</v>
       </c>
       <c r="G10" t="inlineStr" s="7">
         <is>
-          <t>+$36.62 (+5.1%) OTM Buffer 🟢</t>
+          <t>P:+6.0% / C:+4.0% OTM 🟢</t>
         </is>
       </c>
       <c r="H10" s="6">
-        <v>555.0</v>
+        <v>696.0</v>
       </c>
       <c r="I10" s="6">
-        <v>457.0</v>
+        <v>212.0</v>
       </c>
       <c r="J10" s="7">
         <f>H10-I10</f>
-        <v>98.0</v>
+        <v>484.0</v>
       </c>
       <c r="K10" s="7">
         <f>J10*0.5</f>
-        <v>49.0</v>
+        <v>242.0</v>
       </c>
       <c r="L10" s="6">
-        <v>500.0</v>
+        <v>5000.0</v>
       </c>
       <c r="M10" t="inlineStr" s="0">
         <is>
-          <t>Oct 06, 2026 (T-3 DTE)</t>
+          <t>Oct 13, 2026 (T-3 DTE)</t>
         </is>
       </c>
       <c r="N10" t="inlineStr" s="0">
         <is>
-          <t>Oct 09, 2026</t>
+          <t>Oct 16, 2026</t>
         </is>
       </c>
       <c r="O10" t="inlineStr" s="7">
@@ -530,96 +530,291 @@
       </c>
       <c r="C11" t="inlineStr" s="0">
         <is>
-          <t>Tradier Live (#6YB80974)</t>
+          <t>Alpaca Live (#290523608)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="10">
         <is>
-          <t>$425.00P / $420.00P</t>
+          <t>$435.00P / $425.00P</t>
         </is>
       </c>
       <c r="E11" s="0">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F11" s="6">
-        <v>455.62</v>
+        <v>461.59</v>
       </c>
       <c r="G11" t="inlineStr" s="7">
         <is>
-          <t>+$30.62 (+6.7%) OTM Buffer 🟢</t>
+          <t>+$26.59 (+5.8%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H11" s="6">
-        <v>897.0</v>
+        <v>1485.0</v>
       </c>
       <c r="I11" s="6">
-        <v>747.0</v>
+        <v>930.0</v>
       </c>
       <c r="J11" s="7">
         <f>H11-I11</f>
-        <v>150.0</v>
+        <v>555.0</v>
       </c>
       <c r="K11" s="7">
         <f>J11*0.5</f>
+        <v>277.5</v>
+      </c>
+      <c r="L11" s="6">
+        <v>3000.0</v>
+      </c>
+      <c r="M11" t="inlineStr" s="0">
+        <is>
+          <t>Oct 13, 2026 (T-3 DTE)</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr" s="0">
+        <is>
+          <t>Oct 16, 2026</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr" s="7">
+        <is>
+          <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="0">
+        <is>
+          <t>3. Inflation Defense &amp; Hard Assets</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="10">
+        <is>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (#290523608)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="10">
+        <is>
+          <t>$60.00P / $58.00P</t>
+        </is>
+      </c>
+      <c r="E12" s="0">
+        <v>1</v>
+      </c>
+      <c r="F12" s="6">
+        <v>61.96</v>
+      </c>
+      <c r="G12" t="inlineStr" s="7">
+        <is>
+          <t>+$1.96 (+3.2%) OTM Buffer 🟢</t>
+        </is>
+      </c>
+      <c r="H12" s="6">
+        <v>68.0</v>
+      </c>
+      <c r="I12" s="6">
+        <v>32.0</v>
+      </c>
+      <c r="J12" s="7">
+        <f>H12-I12</f>
+        <v>36.0</v>
+      </c>
+      <c r="K12" s="7">
+        <f>J12*0.5</f>
+        <v>18.0</v>
+      </c>
+      <c r="L12" s="6">
+        <v>200.0</v>
+      </c>
+      <c r="M12" t="inlineStr" s="0">
+        <is>
+          <t>Oct 13, 2026 (T-3 DTE)</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr" s="0">
+        <is>
+          <t>Oct 16, 2026</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr" s="7">
+        <is>
+          <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr" s="0">
+        <is>
+          <t>8. Mega-Cap Cloud &amp; Software Platform</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="10">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="0">
+        <is>
+          <t>Tradier Live (#6YB80974)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="10">
+        <is>
+          <t>$685.00P / $680.00P</t>
+        </is>
+      </c>
+      <c r="E13" s="0">
+        <v>1</v>
+      </c>
+      <c r="F13" s="6">
+        <v>736.79</v>
+      </c>
+      <c r="G13" t="inlineStr" s="7">
+        <is>
+          <t>+$51.79 (+7.0%) OTM Buffer 🟢</t>
+        </is>
+      </c>
+      <c r="H13" s="6">
+        <v>555.0</v>
+      </c>
+      <c r="I13" s="6">
+        <v>457.0</v>
+      </c>
+      <c r="J13" s="7">
+        <f>H13-I13</f>
+        <v>98.0</v>
+      </c>
+      <c r="K13" s="7">
+        <f>J13*0.5</f>
+        <v>49.0</v>
+      </c>
+      <c r="L13" s="6">
+        <v>500.0</v>
+      </c>
+      <c r="M13" t="inlineStr" s="0">
+        <is>
+          <t>Oct 06, 2026 (T-3 DTE)</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr" s="0">
+        <is>
+          <t>Oct 09, 2026</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr" s="7">
+        <is>
+          <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr" s="0">
+        <is>
+          <t>1. AI Chips &amp; Hardware</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="10">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="0">
+        <is>
+          <t>Tradier Live (#6YB80974)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="10">
+        <is>
+          <t>$425.00P / $420.00P</t>
+        </is>
+      </c>
+      <c r="E14" s="0">
+        <v>1</v>
+      </c>
+      <c r="F14" s="6">
+        <v>461.59</v>
+      </c>
+      <c r="G14" t="inlineStr" s="7">
+        <is>
+          <t>+$36.59 (+7.9%) OTM Buffer 🟢</t>
+        </is>
+      </c>
+      <c r="H14" s="6">
+        <v>897.0</v>
+      </c>
+      <c r="I14" s="6">
+        <v>747.0</v>
+      </c>
+      <c r="J14" s="7">
+        <f>H14-I14</f>
+        <v>150.0</v>
+      </c>
+      <c r="K14" s="7">
+        <f>J14*0.5</f>
         <v>75.0</v>
       </c>
-      <c r="L11" s="6">
+      <c r="L14" s="6">
         <v>500.0</v>
       </c>
-      <c r="M11" t="inlineStr" s="0">
+      <c r="M14" t="inlineStr" s="0">
         <is>
           <t>Oct 27, 2026 (T-3 DTE)</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr" s="0">
+      <c r="N14" t="inlineStr" s="0">
         <is>
           <t>Oct 30, 2026</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr" s="7">
+      <c r="O14" t="inlineStr" s="7">
         <is>
           <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr" s="5">
+    <row r="15">
+      <c r="A15" t="inlineStr" s="5">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="13">
-        <f>SUM(E8:E11)</f>
-        <v>9</v>
-      </c>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="11">
-        <f>SUM(H8:H11)</f>
-        <v>2546.0</v>
-      </c>
-      <c r="I12" s="11">
-        <f>SUM(I8:I11)</f>
-        <v>1836.0</v>
-      </c>
-      <c r="J12" s="11">
-        <f>SUM(J8:J11)</f>
-        <v>710.0</v>
-      </c>
-      <c r="K12" s="11">
-        <f>SUM(K8:K11)</f>
-        <v>355.0</v>
-      </c>
-      <c r="L12" s="11">
-        <f>SUM(L8:L11)</f>
-        <v>4200.0</v>
-      </c>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" t="inlineStr" s="5">
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="13">
+        <f>SUM(E8:E14)</f>
+        <v>17</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="11">
+        <f>SUM(H8:H14)</f>
+        <v>5705.0</v>
+      </c>
+      <c r="I15" s="11">
+        <f>SUM(I8:I14)</f>
+        <v>3089.0</v>
+      </c>
+      <c r="J15" s="11">
+        <f>SUM(J8:J14)</f>
+        <v>2616.0</v>
+      </c>
+      <c r="K15" s="11">
+        <f>SUM(K8:K14)</f>
+        <v>1308.0</v>
+      </c>
+      <c r="L15" s="11">
+        <f>SUM(L8:L14)</f>
+        <v>21200.0</v>
+      </c>
+      <c r="M15" s="5"/>
+      <c r="N15" s="5"/>
+      <c r="O15" t="inlineStr" s="5">
         <is>
           <t>100% DEFINED RISK PROTECTED ✅</t>
         </is>
@@ -1384,7 +1579,7 @@
       </c>
       <c r="G10" t="inlineStr" s="0">
         <is>
-          <t>14:16:18</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="H10" t="inlineStr" s="0">
@@ -1457,56 +1652,496 @@
       </c>
       <c r="Z10" t="inlineStr" s="0">
         <is>
-          <t>148305471</t>
+          <t>tradier_2026-09-29</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr" s="5">
+      <c r="A11" t="inlineStr" s="0">
+        <is>
+          <t>TRD-20260930-AVGO-335/305</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (#290523608)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="10">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="0">
+        <is>
+          <t>1. AI Chips &amp; Hardware</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="0">
+        <is>
+          <t>Bull Put Spread (335P/305P)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr" s="0">
+        <is>
+          <t>14:36:14</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr" s="0">
+        <is>
+          <t>AVGO261016P00335000</t>
+        </is>
+      </c>
+      <c r="I11" s="6">
+        <v>335.0</v>
+      </c>
+      <c r="J11" t="inlineStr" s="0">
+        <is>
+          <t>AVGO261016P00305000</t>
+        </is>
+      </c>
+      <c r="K11" s="6">
+        <v>305.0</v>
+      </c>
+      <c r="L11" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="M11" s="0">
+        <v>3</v>
+      </c>
+      <c r="N11" s="6">
+        <v>2.89</v>
+      </c>
+      <c r="O11" s="6">
+        <v>867.0</v>
+      </c>
+      <c r="P11" s="6">
+        <v>9000.0</v>
+      </c>
+      <c r="Q11" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S11" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="T11" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="U11" s="6">
+        <v>0.00</v>
+      </c>
+      <c r="V11" s="8">
+        <v>0.0</v>
+      </c>
+      <c r="W11" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="X11" t="inlineStr" s="0">
+        <is>
+          <t>Active with broker (live position)</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr" s="10">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr" s="0">
+        <is>
+          <t>9e306619-a4b3-4116-9ebf-df20c399e587</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="0">
+        <is>
+          <t>TRD-20260930-QQQ-775/800</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (#290523608)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="10">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="0">
+        <is>
+          <t>7. Broad Index &amp; Market Hedging</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr" s="0">
+        <is>
+          <t>Bear Call Spread (775C/800C)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr" s="0">
+        <is>
+          <t>15:13:49</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr" s="0">
+        <is>
+          <t>QQQ261016C00775000</t>
+        </is>
+      </c>
+      <c r="I12" s="6">
+        <v>775.0</v>
+      </c>
+      <c r="J12" t="inlineStr" s="0">
+        <is>
+          <t>QQQ261016C00800000</t>
+        </is>
+      </c>
+      <c r="K12" s="6">
+        <v>800.0</v>
+      </c>
+      <c r="L12" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="M12" s="0">
+        <v>2</v>
+      </c>
+      <c r="N12" s="6">
+        <v>1.42</v>
+      </c>
+      <c r="O12" s="6">
+        <v>284.0</v>
+      </c>
+      <c r="P12" s="6">
+        <v>5000.0</v>
+      </c>
+      <c r="Q12" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S12" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="T12" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="U12" s="6">
+        <v>0.00</v>
+      </c>
+      <c r="V12" s="8">
+        <v>0.0</v>
+      </c>
+      <c r="W12" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="X12" t="inlineStr" s="0">
+        <is>
+          <t>Active with broker (live position)</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr" s="10">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr" s="0">
+        <is>
+          <t>18c2b2bd-a6f0-4943-a0c8-9f12613fbdde</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr" s="0">
+        <is>
+          <t>TRD-20260930-QQQ-700/675</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (#290523608)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="10">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="0">
+        <is>
+          <t>7. Broad Index &amp; Market Hedging</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="0">
+        <is>
+          <t>Bull Put Spread (700P/675P)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr" s="0">
+        <is>
+          <t>15:13:49</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr" s="0">
+        <is>
+          <t>QQQ261016P00700000</t>
+        </is>
+      </c>
+      <c r="I13" s="6">
+        <v>700.0</v>
+      </c>
+      <c r="J13" t="inlineStr" s="0">
+        <is>
+          <t>QQQ261016P00675000</t>
+        </is>
+      </c>
+      <c r="K13" s="6">
+        <v>675.0</v>
+      </c>
+      <c r="L13" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="M13" s="0">
+        <v>2</v>
+      </c>
+      <c r="N13" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="O13" s="6">
+        <v>200.0</v>
+      </c>
+      <c r="P13" s="6">
+        <v>5000.0</v>
+      </c>
+      <c r="Q13" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S13" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="T13" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="U13" s="6">
+        <v>0.00</v>
+      </c>
+      <c r="V13" s="8">
+        <v>0.0</v>
+      </c>
+      <c r="W13" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="X13" t="inlineStr" s="0">
+        <is>
+          <t>Active with broker (live position)</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr" s="10">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr" s="0">
+        <is>
+          <t>a961797c-c700-495c-941e-0e0f66ab5a62</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr" s="0">
+        <is>
+          <t>TRD-20260930-TSM-435/425</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (#290523608)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="10">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="0">
+        <is>
+          <t>1. AI Chips &amp; Hardware</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr" s="0">
+        <is>
+          <t>Bull Put Spread (435P/425P)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr" s="0">
+        <is>
+          <t>14:47:06</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr" s="0">
+        <is>
+          <t>TSM261016P00435000</t>
+        </is>
+      </c>
+      <c r="I14" s="6">
+        <v>435.0</v>
+      </c>
+      <c r="J14" t="inlineStr" s="0">
+        <is>
+          <t>TSM261016P00425000</t>
+        </is>
+      </c>
+      <c r="K14" s="6">
+        <v>425.0</v>
+      </c>
+      <c r="L14" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="M14" s="0">
+        <v>3</v>
+      </c>
+      <c r="N14" s="6">
+        <v>1.85</v>
+      </c>
+      <c r="O14" s="6">
+        <v>555.0</v>
+      </c>
+      <c r="P14" s="6">
+        <v>3000.0</v>
+      </c>
+      <c r="Q14" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S14" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="T14" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="U14" s="6">
+        <v>0.00</v>
+      </c>
+      <c r="V14" s="8">
+        <v>0.0</v>
+      </c>
+      <c r="W14" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="X14" t="inlineStr" s="0">
+        <is>
+          <t>Active with broker (live position)</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr" s="10">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr" s="0">
+        <is>
+          <t>3b71756c-5bf9-4c7e-84b5-813ae535d313</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr" s="5">
         <is>
           <t>TOTALS / RECONCILED</t>
         </is>
       </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="5"/>
-      <c r="L11" s="5"/>
-      <c r="M11" s="13">
-        <f>SUM(M5:M10)</f>
-        <v>11</v>
-      </c>
-      <c r="N11" s="5"/>
-      <c r="O11" s="11">
-        <f>SUM(O5:O10)</f>
-        <v>729.0</v>
-      </c>
-      <c r="P11" s="11">
-        <f>SUM(P5:P10)</f>
-        <v>4500.0</v>
-      </c>
-      <c r="Q11" s="5"/>
-      <c r="R11" s="5"/>
-      <c r="S11" s="5"/>
-      <c r="T11" s="11">
-        <f>SUM(T5:T10)</f>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="13">
+        <f>SUM(M5:M14)</f>
+        <v>21</v>
+      </c>
+      <c r="N15" s="5"/>
+      <c r="O15" s="11">
+        <f>SUM(O5:O14)</f>
+        <v>2635.0</v>
+      </c>
+      <c r="P15" s="11">
+        <f>SUM(P5:P14)</f>
+        <v>26500.0</v>
+      </c>
+      <c r="Q15" s="5"/>
+      <c r="R15" s="5"/>
+      <c r="S15" s="5"/>
+      <c r="T15" s="11">
+        <f>SUM(T5:T14)</f>
         <v>79.0</v>
       </c>
-      <c r="U11" s="11">
-        <f>SUM(U5:U10)</f>
+      <c r="U15" s="11">
+        <f>SUM(U5:U14)</f>
         <v>-60.0</v>
       </c>
-      <c r="V11" s="5"/>
-      <c r="W11" s="5"/>
-      <c r="X11" s="5"/>
-      <c r="Y11" s="5"/>
-      <c r="Z11" s="5"/>
+      <c r="V15" s="5"/>
+      <c r="W15" s="5"/>
+      <c r="X15" s="5"/>
+      <c r="Y15" s="5"/>
+      <c r="Z15" s="5"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
sync: reconcile active trades and live transaction journal post QQQ call wing harvest
</commit_message>
<xml_diff>
--- a/SkonVault_Live_Transaction_Journal.xlsx
+++ b/SkonVault_Live_Transaction_Journal.xlsx
@@ -184,7 +184,7 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
         <is>
-          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-09-30 22:53 ICT</t>
+          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-10-01 21:23 ICT</t>
         </is>
       </c>
     </row>
@@ -222,26 +222,26 @@
     </row>
     <row r="5">
       <c r="A5" s="6">
-        <v>34634.77</v>
+        <v>34388.52</v>
       </c>
       <c r="C5" s="6">
         <v>11249.0</v>
       </c>
       <c r="E5" s="7">
-        <f>J15</f>
-        <v>2616.0</v>
+        <f>J14</f>
+        <v>2234.0</v>
       </c>
       <c r="G5" s="7">
-        <f>K15</f>
-        <v>1308.0</v>
+        <f>K14</f>
+        <v>1117.0</v>
       </c>
       <c r="I5" s="6">
-        <f>L15</f>
-        <v>21200.0</v>
+        <f>L14</f>
+        <v>20700.0</v>
       </c>
       <c r="K5" t="inlineStr" s="10">
         <is>
-          <t>108.2% CASH RESERVE (≥35% FLOOR) 🟢</t>
+          <t>109.4% CASH RESERVE (≥35% FLOOR) 🟢</t>
         </is>
       </c>
     </row>
@@ -347,11 +347,11 @@
         <v>3</v>
       </c>
       <c r="F8" s="6">
-        <v>354.2875</v>
+        <v>347.99</v>
       </c>
       <c r="G8" t="inlineStr" s="7">
         <is>
-          <t>+$19.29 (+5.4%) OTM Buffer 🟢</t>
+          <t>+$12.99 (+3.7%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H8" s="6">
@@ -412,11 +412,11 @@
         <v>6</v>
       </c>
       <c r="F9" s="6">
-        <v>231.05</v>
+        <v>229.68</v>
       </c>
       <c r="G9" t="inlineStr" s="7">
         <is>
-          <t>+$11.05 (+4.8%) OTM Buffer 🟢</t>
+          <t>+$9.68 (+4.2%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H9" s="6">
@@ -470,33 +470,33 @@
       </c>
       <c r="D10" t="inlineStr" s="10">
         <is>
-          <t>$700P/$675P &amp; $775C/$800C (IC)</t>
+          <t>$700.00P / $675.00P</t>
         </is>
       </c>
       <c r="E10" s="0">
         <v>2</v>
       </c>
       <c r="F10" s="6">
-        <v>745.05</v>
+        <v>738.13</v>
       </c>
       <c r="G10" t="inlineStr" s="7">
         <is>
-          <t>P:+6.0% / C:+4.0% OTM 🟢</t>
+          <t>+$38.13 (+5.2%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H10" s="6">
-        <v>696.0</v>
+        <v>368.0</v>
       </c>
       <c r="I10" s="6">
-        <v>212.0</v>
+        <v>168.0</v>
       </c>
       <c r="J10" s="7">
         <f>H10-I10</f>
-        <v>484.0</v>
+        <v>200.0</v>
       </c>
       <c r="K10" s="7">
         <f>J10*0.5</f>
-        <v>242.0</v>
+        <v>100.0</v>
       </c>
       <c r="L10" s="6">
         <v>5000.0</v>
@@ -542,11 +542,11 @@
         <v>3</v>
       </c>
       <c r="F11" s="6">
-        <v>461.59</v>
+        <v>455.56</v>
       </c>
       <c r="G11" t="inlineStr" s="7">
         <is>
-          <t>+$26.59 (+5.8%) OTM Buffer 🟢</t>
+          <t>+$20.56 (+4.5%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H11" s="6">
@@ -607,11 +607,11 @@
         <v>1</v>
       </c>
       <c r="F12" s="6">
-        <v>61.96</v>
+        <v>62.06</v>
       </c>
       <c r="G12" t="inlineStr" s="7">
         <is>
-          <t>+$1.96 (+3.2%) OTM Buffer 🟢</t>
+          <t>+$2.06 (+3.3%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H12" s="6">
@@ -650,12 +650,12 @@
     <row r="13">
       <c r="A13" t="inlineStr" s="0">
         <is>
-          <t>8. Mega-Cap Cloud &amp; Software Platform</t>
+          <t>1. AI Chips &amp; Hardware</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="10">
         <is>
-          <t>META</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="0">
@@ -665,45 +665,45 @@
       </c>
       <c r="D13" t="inlineStr" s="10">
         <is>
-          <t>$685.00P / $680.00P</t>
+          <t>$425.00P / $420.00P</t>
         </is>
       </c>
       <c r="E13" s="0">
         <v>1</v>
       </c>
       <c r="F13" s="6">
-        <v>736.79</v>
+        <v>455.56</v>
       </c>
       <c r="G13" t="inlineStr" s="7">
         <is>
-          <t>+$51.79 (+7.0%) OTM Buffer 🟢</t>
+          <t>+$30.56 (+6.7%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H13" s="6">
-        <v>555.0</v>
+        <v>897.0</v>
       </c>
       <c r="I13" s="6">
-        <v>457.0</v>
+        <v>747.0</v>
       </c>
       <c r="J13" s="7">
         <f>H13-I13</f>
-        <v>98.0</v>
+        <v>150.0</v>
       </c>
       <c r="K13" s="7">
         <f>J13*0.5</f>
-        <v>49.0</v>
+        <v>75.0</v>
       </c>
       <c r="L13" s="6">
         <v>500.0</v>
       </c>
       <c r="M13" t="inlineStr" s="0">
         <is>
-          <t>Oct 06, 2026 (T-3 DTE)</t>
+          <t>Oct 27, 2026 (T-3 DTE)</t>
         </is>
       </c>
       <c r="N13" t="inlineStr" s="0">
         <is>
-          <t>Oct 09, 2026</t>
+          <t>Oct 30, 2026</t>
         </is>
       </c>
       <c r="O13" t="inlineStr" s="7">
@@ -713,108 +713,43 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr" s="0">
-        <is>
-          <t>1. AI Chips &amp; Hardware</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr" s="10">
-        <is>
-          <t>TSM</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr" s="0">
-        <is>
-          <t>Tradier Live (#6YB80974)</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr" s="10">
-        <is>
-          <t>$425.00P / $420.00P</t>
-        </is>
-      </c>
-      <c r="E14" s="0">
-        <v>1</v>
-      </c>
-      <c r="F14" s="6">
-        <v>461.59</v>
-      </c>
-      <c r="G14" t="inlineStr" s="7">
-        <is>
-          <t>+$36.59 (+7.9%) OTM Buffer 🟢</t>
-        </is>
-      </c>
-      <c r="H14" s="6">
-        <v>897.0</v>
-      </c>
-      <c r="I14" s="6">
-        <v>747.0</v>
-      </c>
-      <c r="J14" s="7">
-        <f>H14-I14</f>
-        <v>150.0</v>
-      </c>
-      <c r="K14" s="7">
-        <f>J14*0.5</f>
-        <v>75.0</v>
-      </c>
-      <c r="L14" s="6">
-        <v>500.0</v>
-      </c>
-      <c r="M14" t="inlineStr" s="0">
-        <is>
-          <t>Oct 27, 2026 (T-3 DTE)</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr" s="0">
-        <is>
-          <t>Oct 30, 2026</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr" s="7">
-        <is>
-          <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr" s="5">
+      <c r="A14" t="inlineStr" s="5">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="13">
-        <f>SUM(E8:E14)</f>
-        <v>17</v>
-      </c>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="11">
-        <f>SUM(H8:H14)</f>
-        <v>5705.0</v>
-      </c>
-      <c r="I15" s="11">
-        <f>SUM(I8:I14)</f>
-        <v>3089.0</v>
-      </c>
-      <c r="J15" s="11">
-        <f>SUM(J8:J14)</f>
-        <v>2616.0</v>
-      </c>
-      <c r="K15" s="11">
-        <f>SUM(K8:K14)</f>
-        <v>1308.0</v>
-      </c>
-      <c r="L15" s="11">
-        <f>SUM(L8:L14)</f>
-        <v>21200.0</v>
-      </c>
-      <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-      <c r="O15" t="inlineStr" s="5">
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="13">
+        <f>SUM(E8:E13)</f>
+        <v>16</v>
+      </c>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="11">
+        <f>SUM(H8:H13)</f>
+        <v>4822.0</v>
+      </c>
+      <c r="I14" s="11">
+        <f>SUM(I8:I13)</f>
+        <v>2588.0</v>
+      </c>
+      <c r="J14" s="11">
+        <f>SUM(J8:J13)</f>
+        <v>2234.0</v>
+      </c>
+      <c r="K14" s="11">
+        <f>SUM(K8:K13)</f>
+        <v>1117.0</v>
+      </c>
+      <c r="L14" s="11">
+        <f>SUM(L8:L13)</f>
+        <v>20700.0</v>
+      </c>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" t="inlineStr" s="5">
         <is>
           <t>100% DEFINED RISK PROTECTED ✅</t>
         </is>
@@ -1617,37 +1552,39 @@
       </c>
       <c r="Q10" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R10" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="S10" s="6">
-        <v>0.0</v>
+        <v>0.67</v>
       </c>
       <c r="T10" s="6">
-        <v>0.0</v>
-      </c>
-      <c r="U10" s="6">
-        <v>0.00</v>
+        <v>67.0</v>
+      </c>
+      <c r="U10" s="7">
+        <f>O10-T10</f>
+        <v>31.0</v>
       </c>
       <c r="V10" s="8">
-        <v>0.0</v>
+        <f>IF(P10&gt;0,U10/P10,0)</f>
+        <v>0.062</v>
       </c>
       <c r="W10" s="0">
-        <v>0.0</v>
+        <v>24.0</v>
       </c>
       <c r="X10" t="inlineStr" s="0">
         <is>
-          <t>Active with broker (live position)</t>
+          <t>Take-profit close (verified fill)</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr" s="10">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED_HARVESTED</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr" s="0">
@@ -1837,37 +1774,39 @@
       </c>
       <c r="Q12" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R12" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>14:20:26</t>
         </is>
       </c>
       <c r="S12" s="6">
-        <v>0.0</v>
+        <v>0.89</v>
       </c>
       <c r="T12" s="6">
-        <v>0.0</v>
-      </c>
-      <c r="U12" s="6">
-        <v>0.00</v>
+        <v>178.0</v>
+      </c>
+      <c r="U12" s="7">
+        <f>O12-T12</f>
+        <v>106.0</v>
       </c>
       <c r="V12" s="8">
-        <v>0.0</v>
+        <f>IF(P12&gt;0,U12/P12,0)</f>
+        <v>0.0212</v>
       </c>
       <c r="W12" s="0">
-        <v>0.0</v>
+        <v>23.1</v>
       </c>
       <c r="X12" t="inlineStr" s="0">
         <is>
-          <t>Active with broker (live position)</t>
+          <t>Take-profit close (verified fill) — rolled / re-entered 2x</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr" s="10">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED_HARVESTED</t>
         </is>
       </c>
       <c r="Z12" t="inlineStr" s="0">
@@ -2131,11 +2070,11 @@
       <c r="S15" s="5"/>
       <c r="T15" s="11">
         <f>SUM(T5:T14)</f>
-        <v>79.0</v>
+        <v>324.0</v>
       </c>
       <c r="U15" s="11">
         <f>SUM(U5:U14)</f>
-        <v>-60.0</v>
+        <v>77.0</v>
       </c>
       <c r="V15" s="5"/>
       <c r="W15" s="5"/>
@@ -2345,37 +2284,143 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr" s="5">
+      <c r="A7" t="inlineStr" s="0">
+        <is>
+          <t>TAX-20260929-META-685/680</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="0">
+        <is>
+          <t>Tradier (Apex Clearing Corp)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="0">
+        <is>
+          <t>6YB80974</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="10">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="F7" s="6">
+        <v>98.0</v>
+      </c>
+      <c r="G7" s="6">
+        <v>67.0</v>
+      </c>
+      <c r="H7" s="7">
+        <f>F7-G7</f>
+        <v>31.0</v>
+      </c>
+      <c r="I7" s="6">
+        <v>36.5</v>
+      </c>
+      <c r="J7" s="9">
+        <f>IF(H7&gt;0,H7*I7,0)</f>
+        <v>1131.5</v>
+      </c>
+      <c r="K7" s="9">
+        <f>J7</f>
+        <v>1131.5</v>
+      </c>
+      <c r="L7" t="inlineStr" s="0">
+        <is>
+          <t>tradier_2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="0">
+        <is>
+          <t>TAX-20260930-QQQ-775/800</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Securities LLC</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="0">
+        <is>
+          <t>290523608</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="10">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="F8" s="6">
+        <v>284.0</v>
+      </c>
+      <c r="G8" s="6">
+        <v>178.0</v>
+      </c>
+      <c r="H8" s="7">
+        <f>F8-G8</f>
+        <v>106.0</v>
+      </c>
+      <c r="I8" s="6">
+        <v>36.5</v>
+      </c>
+      <c r="J8" s="9">
+        <f>IF(H8&gt;0,H8*I8,0)</f>
+        <v>3869.0</v>
+      </c>
+      <c r="K8" s="9">
+        <f>J8</f>
+        <v>3869.0</v>
+      </c>
+      <c r="L8" t="inlineStr" s="0">
+        <is>
+          <t>18c2b2bd-a6f0-4943-a0c8-9f12613fbdde</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="5">
         <is>
           <t>TOTAL CLOSED REVENUE</t>
         </is>
       </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="11">
-        <f>SUM(F5:F6)</f>
-        <v>19.0</v>
-      </c>
-      <c r="G7" s="11">
-        <f>SUM(G5:G6)</f>
-        <v>79.0</v>
-      </c>
-      <c r="H7" s="11">
-        <f>SUM(H5:H6)</f>
-        <v>-60.0</v>
-      </c>
-      <c r="I7" s="5"/>
-      <c r="J7" s="12">
-        <f>SUM(J5:J6)</f>
-        <v>0.0</v>
-      </c>
-      <c r="K7" s="12">
-        <f>SUM(K5:K6)</f>
-        <v>0.0</v>
-      </c>
-      <c r="L7" t="inlineStr" s="5">
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="11">
+        <f>SUM(F5:F8)</f>
+        <v>401.0</v>
+      </c>
+      <c r="G9" s="11">
+        <f>SUM(G5:G8)</f>
+        <v>324.0</v>
+      </c>
+      <c r="H9" s="11">
+        <f>SUM(H5:H8)</f>
+        <v>77.0</v>
+      </c>
+      <c r="I9" s="5"/>
+      <c r="J9" s="12">
+        <f>SUM(J5:J8)</f>
+        <v>5000.5</v>
+      </c>
+      <c r="K9" s="12">
+        <f>SUM(K5:K8)</f>
+        <v>5000.5</v>
+      </c>
+      <c r="L9" t="inlineStr" s="5">
         <is>
           <t>AUDITED COMPLIANT ✅</t>
         </is>

</xml_diff>

<commit_message>
feat(tradier): enable RULE-081 autonomous fallback relay and RULE-098 dual dispatch for Tradier Live
</commit_message>
<xml_diff>
--- a/SkonVault_Live_Transaction_Journal.xlsx
+++ b/SkonVault_Live_Transaction_Journal.xlsx
@@ -184,7 +184,7 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
         <is>
-          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-10-01 21:23 ICT</t>
+          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-10-02 09:04 ICT</t>
         </is>
       </c>
     </row>
@@ -222,26 +222,26 @@
     </row>
     <row r="5">
       <c r="A5" s="6">
-        <v>34388.52</v>
+        <v>33986.02</v>
       </c>
       <c r="C5" s="6">
         <v>11249.0</v>
       </c>
       <c r="E5" s="7">
-        <f>J14</f>
-        <v>2234.0</v>
+        <f>J13</f>
+        <v>1808.0</v>
       </c>
       <c r="G5" s="7">
-        <f>K14</f>
-        <v>1117.0</v>
+        <f>K13</f>
+        <v>904.0</v>
       </c>
       <c r="I5" s="6">
-        <f>L14</f>
-        <v>20700.0</v>
+        <f>L13</f>
+        <v>17700.0</v>
       </c>
       <c r="K5" t="inlineStr" s="10">
         <is>
-          <t>109.4% CASH RESERVE (≥35% FLOOR) 🟢</t>
+          <t>107.7% CASH RESERVE (≥35% FLOOR) 🟢</t>
         </is>
       </c>
     </row>
@@ -347,11 +347,11 @@
         <v>3</v>
       </c>
       <c r="F8" s="6">
-        <v>347.99</v>
+        <v>343.64</v>
       </c>
       <c r="G8" t="inlineStr" s="7">
         <is>
-          <t>+$12.99 (+3.7%) OTM Buffer 🟢</t>
+          <t>+$8.64 (+2.5%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H8" s="6">
@@ -390,12 +390,12 @@
     <row r="9">
       <c r="A9" t="inlineStr" s="0">
         <is>
-          <t>1. AI Chips &amp; Hardware</t>
+          <t>7. Broad Index &amp; Market Hedging</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="10">
         <is>
-          <t>NVDA</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="0">
@@ -405,45 +405,45 @@
       </c>
       <c r="D9" t="inlineStr" s="10">
         <is>
-          <t>$220.00P / $215.00P</t>
+          <t>$700.00P / $675.00P</t>
         </is>
       </c>
       <c r="E9" s="0">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F9" s="6">
-        <v>229.68</v>
+        <v>742.03</v>
       </c>
       <c r="G9" t="inlineStr" s="7">
         <is>
-          <t>+$9.68 (+4.2%) OTM Buffer 🟢</t>
+          <t>+$42.03 (+5.7%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H9" s="6">
-        <v>1026.0</v>
+        <v>368.0</v>
       </c>
       <c r="I9" s="6">
-        <v>600.0</v>
+        <v>168.0</v>
       </c>
       <c r="J9" s="7">
         <f>H9-I9</f>
-        <v>426.0</v>
+        <v>200.0</v>
       </c>
       <c r="K9" s="7">
         <f>J9*0.5</f>
-        <v>213.0</v>
+        <v>100.0</v>
       </c>
       <c r="L9" s="6">
-        <v>3000.0</v>
+        <v>5000.0</v>
       </c>
       <c r="M9" t="inlineStr" s="0">
         <is>
-          <t>Oct 07, 2026 (T-3 DTE)</t>
+          <t>Oct 13, 2026 (T-3 DTE)</t>
         </is>
       </c>
       <c r="N9" t="inlineStr" s="0">
         <is>
-          <t>Oct 12, 2026</t>
+          <t>Oct 16, 2026</t>
         </is>
       </c>
       <c r="O9" t="inlineStr" s="7">
@@ -455,12 +455,12 @@
     <row r="10">
       <c r="A10" t="inlineStr" s="0">
         <is>
-          <t>7. Broad Index &amp; Market Hedging</t>
+          <t>1. AI Chips &amp; Hardware</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="10">
         <is>
-          <t>QQQ</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="0">
@@ -470,36 +470,36 @@
       </c>
       <c r="D10" t="inlineStr" s="10">
         <is>
-          <t>$700.00P / $675.00P</t>
+          <t>$435.00P / $425.00P</t>
         </is>
       </c>
       <c r="E10" s="0">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" s="6">
-        <v>738.13</v>
+        <v>459.2</v>
       </c>
       <c r="G10" t="inlineStr" s="7">
         <is>
-          <t>+$38.13 (+5.2%) OTM Buffer 🟢</t>
+          <t>+$24.20 (+5.3%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H10" s="6">
-        <v>368.0</v>
+        <v>1485.0</v>
       </c>
       <c r="I10" s="6">
-        <v>168.0</v>
+        <v>930.0</v>
       </c>
       <c r="J10" s="7">
         <f>H10-I10</f>
-        <v>200.0</v>
+        <v>555.0</v>
       </c>
       <c r="K10" s="7">
         <f>J10*0.5</f>
-        <v>100.0</v>
+        <v>277.5</v>
       </c>
       <c r="L10" s="6">
-        <v>5000.0</v>
+        <v>3000.0</v>
       </c>
       <c r="M10" t="inlineStr" s="0">
         <is>
@@ -520,12 +520,12 @@
     <row r="11">
       <c r="A11" t="inlineStr" s="0">
         <is>
-          <t>1. AI Chips &amp; Hardware</t>
+          <t>3. Inflation Defense &amp; Hard Assets</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="10">
         <is>
-          <t>TSM</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="0">
@@ -535,36 +535,36 @@
       </c>
       <c r="D11" t="inlineStr" s="10">
         <is>
-          <t>$435.00P / $425.00P</t>
+          <t>$60.00P / $58.00P</t>
         </is>
       </c>
       <c r="E11" s="0">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F11" s="6">
-        <v>455.56</v>
+        <v>62.7</v>
       </c>
       <c r="G11" t="inlineStr" s="7">
         <is>
-          <t>+$20.56 (+4.5%) OTM Buffer 🟢</t>
+          <t>+$2.70 (+4.3%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H11" s="6">
-        <v>1485.0</v>
+        <v>68.0</v>
       </c>
       <c r="I11" s="6">
-        <v>930.0</v>
+        <v>32.0</v>
       </c>
       <c r="J11" s="7">
         <f>H11-I11</f>
-        <v>555.0</v>
+        <v>36.0</v>
       </c>
       <c r="K11" s="7">
         <f>J11*0.5</f>
-        <v>277.5</v>
+        <v>18.0</v>
       </c>
       <c r="L11" s="6">
-        <v>3000.0</v>
+        <v>200.0</v>
       </c>
       <c r="M11" t="inlineStr" s="0">
         <is>
@@ -585,60 +585,60 @@
     <row r="12">
       <c r="A12" t="inlineStr" s="0">
         <is>
-          <t>3. Inflation Defense &amp; Hard Assets</t>
+          <t>1. AI Chips &amp; Hardware</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="10">
         <is>
-          <t>XLE</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="0">
         <is>
-          <t>Alpaca Live (#290523608)</t>
+          <t>Tradier Live (#6YB80974)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="10">
         <is>
-          <t>$60.00P / $58.00P</t>
+          <t>$425.00P / $420.00P</t>
         </is>
       </c>
       <c r="E12" s="0">
         <v>1</v>
       </c>
       <c r="F12" s="6">
-        <v>62.06</v>
+        <v>459.2</v>
       </c>
       <c r="G12" t="inlineStr" s="7">
         <is>
-          <t>+$2.06 (+3.3%) OTM Buffer 🟢</t>
+          <t>+$34.20 (+7.4%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H12" s="6">
-        <v>68.0</v>
+        <v>897.0</v>
       </c>
       <c r="I12" s="6">
-        <v>32.0</v>
+        <v>747.0</v>
       </c>
       <c r="J12" s="7">
         <f>H12-I12</f>
-        <v>36.0</v>
+        <v>150.0</v>
       </c>
       <c r="K12" s="7">
         <f>J12*0.5</f>
-        <v>18.0</v>
+        <v>75.0</v>
       </c>
       <c r="L12" s="6">
-        <v>200.0</v>
+        <v>500.0</v>
       </c>
       <c r="M12" t="inlineStr" s="0">
         <is>
-          <t>Oct 13, 2026 (T-3 DTE)</t>
+          <t>Oct 27, 2026 (T-3 DTE)</t>
         </is>
       </c>
       <c r="N12" t="inlineStr" s="0">
         <is>
-          <t>Oct 16, 2026</t>
+          <t>Oct 30, 2026</t>
         </is>
       </c>
       <c r="O12" t="inlineStr" s="7">
@@ -648,108 +648,43 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr" s="0">
-        <is>
-          <t>1. AI Chips &amp; Hardware</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr" s="10">
-        <is>
-          <t>TSM</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr" s="0">
-        <is>
-          <t>Tradier Live (#6YB80974)</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr" s="10">
-        <is>
-          <t>$425.00P / $420.00P</t>
-        </is>
-      </c>
-      <c r="E13" s="0">
-        <v>1</v>
-      </c>
-      <c r="F13" s="6">
-        <v>455.56</v>
-      </c>
-      <c r="G13" t="inlineStr" s="7">
-        <is>
-          <t>+$30.56 (+6.7%) OTM Buffer 🟢</t>
-        </is>
-      </c>
-      <c r="H13" s="6">
-        <v>897.0</v>
-      </c>
-      <c r="I13" s="6">
-        <v>747.0</v>
-      </c>
-      <c r="J13" s="7">
-        <f>H13-I13</f>
-        <v>150.0</v>
-      </c>
-      <c r="K13" s="7">
-        <f>J13*0.5</f>
-        <v>75.0</v>
-      </c>
-      <c r="L13" s="6">
-        <v>500.0</v>
-      </c>
-      <c r="M13" t="inlineStr" s="0">
-        <is>
-          <t>Oct 27, 2026 (T-3 DTE)</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr" s="0">
-        <is>
-          <t>Oct 30, 2026</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr" s="7">
-        <is>
-          <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr" s="5">
+      <c r="A13" t="inlineStr" s="5">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="13">
-        <f>SUM(E8:E13)</f>
-        <v>16</v>
-      </c>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="11">
-        <f>SUM(H8:H13)</f>
-        <v>4822.0</v>
-      </c>
-      <c r="I14" s="11">
-        <f>SUM(I8:I13)</f>
-        <v>2588.0</v>
-      </c>
-      <c r="J14" s="11">
-        <f>SUM(J8:J13)</f>
-        <v>2234.0</v>
-      </c>
-      <c r="K14" s="11">
-        <f>SUM(K8:K13)</f>
-        <v>1117.0</v>
-      </c>
-      <c r="L14" s="11">
-        <f>SUM(L8:L13)</f>
-        <v>20700.0</v>
-      </c>
-      <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" t="inlineStr" s="5">
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="13">
+        <f>SUM(E8:E12)</f>
+        <v>10</v>
+      </c>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="11">
+        <f>SUM(H8:H12)</f>
+        <v>3796.0</v>
+      </c>
+      <c r="I13" s="11">
+        <f>SUM(I8:I12)</f>
+        <v>1988.0</v>
+      </c>
+      <c r="J13" s="11">
+        <f>SUM(J8:J12)</f>
+        <v>1808.0</v>
+      </c>
+      <c r="K13" s="11">
+        <f>SUM(K8:K12)</f>
+        <v>904.0</v>
+      </c>
+      <c r="L13" s="11">
+        <f>SUM(L8:L12)</f>
+        <v>17700.0</v>
+      </c>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" t="inlineStr" s="5">
         <is>
           <t>100% DEFINED RISK PROTECTED ✅</t>
         </is>
@@ -1332,37 +1267,39 @@
       </c>
       <c r="Q8" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R8" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>19:55:15</t>
         </is>
       </c>
       <c r="S8" s="6">
-        <v>0.0</v>
+        <v>0.67</v>
       </c>
       <c r="T8" s="6">
-        <v>0.0</v>
-      </c>
-      <c r="U8" s="6">
-        <v>0.00</v>
+        <v>402.0</v>
+      </c>
+      <c r="U8" s="7">
+        <f>O8-T8</f>
+        <v>24.0</v>
       </c>
       <c r="V8" s="8">
-        <v>0.0</v>
+        <f>IF(P8&gt;0,U8/P8,0)</f>
+        <v>0.008</v>
       </c>
       <c r="W8" s="0">
-        <v>0.0</v>
+        <v>77.6</v>
       </c>
       <c r="X8" t="inlineStr" s="0">
         <is>
-          <t>Active with broker (live position)</t>
+          <t>Take-profit close (verified fill)</t>
         </is>
       </c>
       <c r="Y8" t="inlineStr" s="10">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED_HARVESTED</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr" s="0">
@@ -2070,11 +2007,11 @@
       <c r="S15" s="5"/>
       <c r="T15" s="11">
         <f>SUM(T5:T14)</f>
-        <v>324.0</v>
+        <v>726.0</v>
       </c>
       <c r="U15" s="11">
         <f>SUM(U5:U14)</f>
-        <v>77.0</v>
+        <v>101.0</v>
       </c>
       <c r="V15" s="5"/>
       <c r="W15" s="5"/>
@@ -2286,141 +2223,194 @@
     <row r="7">
       <c r="A7" t="inlineStr" s="0">
         <is>
-          <t>TAX-20260929-META-685/680</t>
+          <t>TAX-20260928-NVDA-220/215</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="0">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="0">
         <is>
-          <t>Tradier (Apex Clearing Corp)</t>
+          <t>Alpaca Securities LLC</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="0">
         <is>
-          <t>6YB80974</t>
+          <t>290523608</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="10">
         <is>
-          <t>META</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="F7" s="6">
-        <v>98.0</v>
+        <v>426.0</v>
       </c>
       <c r="G7" s="6">
-        <v>67.0</v>
+        <v>402.0</v>
       </c>
       <c r="H7" s="7">
         <f>F7-G7</f>
-        <v>31.0</v>
+        <v>24.0</v>
       </c>
       <c r="I7" s="6">
         <v>36.5</v>
       </c>
       <c r="J7" s="9">
         <f>IF(H7&gt;0,H7*I7,0)</f>
-        <v>1131.5</v>
+        <v>876.0</v>
       </c>
       <c r="K7" s="9">
         <f>J7</f>
-        <v>1131.5</v>
+        <v>876.0</v>
       </c>
       <c r="L7" t="inlineStr" s="0">
         <is>
-          <t>tradier_2026-09-29</t>
+          <t>b62cee06-2bd9-43c4-a8ce-53385fad4b19</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr" s="0">
         <is>
-          <t>TAX-20260930-QQQ-775/800</t>
+          <t>TAX-20260929-META-685/680</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="0">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t>Alpaca Securities LLC</t>
+          <t>Tradier (Apex Clearing Corp)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="0">
         <is>
-          <t>290523608</t>
+          <t>6YB80974</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="10">
         <is>
-          <t>QQQ</t>
+          <t>META</t>
         </is>
       </c>
       <c r="F8" s="6">
-        <v>284.0</v>
+        <v>98.0</v>
       </c>
       <c r="G8" s="6">
-        <v>178.0</v>
+        <v>67.0</v>
       </c>
       <c r="H8" s="7">
         <f>F8-G8</f>
-        <v>106.0</v>
+        <v>31.0</v>
       </c>
       <c r="I8" s="6">
         <v>36.5</v>
       </c>
       <c r="J8" s="9">
         <f>IF(H8&gt;0,H8*I8,0)</f>
-        <v>3869.0</v>
+        <v>1131.5</v>
       </c>
       <c r="K8" s="9">
         <f>J8</f>
+        <v>1131.5</v>
+      </c>
+      <c r="L8" t="inlineStr" s="0">
+        <is>
+          <t>tradier_2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="0">
+        <is>
+          <t>TAX-20260930-QQQ-775/800</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Securities LLC</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="0">
+        <is>
+          <t>290523608</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="10">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="F9" s="6">
+        <v>284.0</v>
+      </c>
+      <c r="G9" s="6">
+        <v>178.0</v>
+      </c>
+      <c r="H9" s="7">
+        <f>F9-G9</f>
+        <v>106.0</v>
+      </c>
+      <c r="I9" s="6">
+        <v>36.5</v>
+      </c>
+      <c r="J9" s="9">
+        <f>IF(H9&gt;0,H9*I9,0)</f>
         <v>3869.0</v>
       </c>
-      <c r="L8" t="inlineStr" s="0">
+      <c r="K9" s="9">
+        <f>J9</f>
+        <v>3869.0</v>
+      </c>
+      <c r="L9" t="inlineStr" s="0">
         <is>
           <t>18c2b2bd-a6f0-4943-a0c8-9f12613fbdde</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr" s="5">
+    <row r="10">
+      <c r="A10" t="inlineStr" s="5">
         <is>
           <t>TOTAL CLOSED REVENUE</t>
         </is>
       </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="11">
-        <f>SUM(F5:F8)</f>
-        <v>401.0</v>
-      </c>
-      <c r="G9" s="11">
-        <f>SUM(G5:G8)</f>
-        <v>324.0</v>
-      </c>
-      <c r="H9" s="11">
-        <f>SUM(H5:H8)</f>
-        <v>77.0</v>
-      </c>
-      <c r="I9" s="5"/>
-      <c r="J9" s="12">
-        <f>SUM(J5:J8)</f>
-        <v>5000.5</v>
-      </c>
-      <c r="K9" s="12">
-        <f>SUM(K5:K8)</f>
-        <v>5000.5</v>
-      </c>
-      <c r="L9" t="inlineStr" s="5">
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="11">
+        <f>SUM(F5:F9)</f>
+        <v>827.0</v>
+      </c>
+      <c r="G10" s="11">
+        <f>SUM(G5:G9)</f>
+        <v>726.0</v>
+      </c>
+      <c r="H10" s="11">
+        <f>SUM(H5:H9)</f>
+        <v>101.0</v>
+      </c>
+      <c r="I10" s="5"/>
+      <c r="J10" s="12">
+        <f>SUM(J5:J9)</f>
+        <v>5876.5</v>
+      </c>
+      <c r="K10" s="12">
+        <f>SUM(K5:K9)</f>
+        <v>5876.5</v>
+      </c>
+      <c r="L10" t="inlineStr" s="5">
         <is>
           <t>AUDITED COMPLIANT ✅</t>
         </is>

</xml_diff>

<commit_message>
fix(journal): cycle-matching spread reconstruction and restore Wise_Capital_Deposits sheet
</commit_message>
<xml_diff>
--- a/SkonVault_Live_Transaction_Journal.xlsx
+++ b/SkonVault_Live_Transaction_Journal.xlsx
@@ -4,7 +4,8 @@
   <sheets>
     <sheet name="Active_Spread_Income_Tracker" sheetId="1" r:id="rId1"/>
     <sheet name="Internal_PnL_Journal" sheetId="2" r:id="rId2"/>
-    <sheet name="External_PnL_Revenue_Report" sheetId="3" r:id="rId3"/>
+    <sheet name="Wise_Capital_Deposits" sheetId="3" r:id="rId3"/>
+    <sheet name="External_PnL_Revenue_Report" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -184,7 +185,7 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
         <is>
-          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-10-02 09:04 ICT</t>
+          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-10-03 06:43 ICT</t>
         </is>
       </c>
     </row>
@@ -222,26 +223,26 @@
     </row>
     <row r="5">
       <c r="A5" s="6">
-        <v>33986.02</v>
+        <v>33271.32</v>
       </c>
       <c r="C5" s="6">
-        <v>11249.0</v>
+        <v>11427.61</v>
       </c>
       <c r="E5" s="7">
-        <f>J13</f>
-        <v>1808.0</v>
+        <f>J10</f>
+        <v>559.0</v>
       </c>
       <c r="G5" s="7">
-        <f>K13</f>
-        <v>904.0</v>
+        <f>K10</f>
+        <v>279.5</v>
       </c>
       <c r="I5" s="6">
-        <f>L13</f>
-        <v>17700.0</v>
+        <f>L10</f>
+        <v>3500.0</v>
       </c>
       <c r="K5" t="inlineStr" s="10">
         <is>
-          <t>107.7% CASH RESERVE (≥35% FLOOR) 🟢</t>
+          <t>101.9% CASH RESERVE (≥35% FLOOR) 🟢</t>
         </is>
       </c>
     </row>
@@ -330,7 +331,7 @@
       </c>
       <c r="B8" t="inlineStr" s="10">
         <is>
-          <t>AVGO</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="0">
@@ -340,36 +341,36 @@
       </c>
       <c r="D8" t="inlineStr" s="10">
         <is>
-          <t>$335.00P / $305.00P</t>
+          <t>$445.00P / $435.00P</t>
         </is>
       </c>
       <c r="E8" s="0">
         <v>3</v>
       </c>
       <c r="F8" s="6">
-        <v>343.64</v>
+        <v>472.78</v>
       </c>
       <c r="G8" t="inlineStr" s="7">
         <is>
-          <t>+$8.64 (+2.5%) OTM Buffer 🟢</t>
+          <t>+$27.78 (+5.9%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H8" s="6">
-        <v>978.0</v>
+        <v>1170.0</v>
       </c>
       <c r="I8" s="6">
-        <v>111.0</v>
+        <v>711.0</v>
       </c>
       <c r="J8" s="7">
         <f>H8-I8</f>
-        <v>867.0</v>
+        <v>459.0</v>
       </c>
       <c r="K8" s="7">
         <f>J8*0.5</f>
-        <v>433.5</v>
+        <v>229.5</v>
       </c>
       <c r="L8" s="6">
-        <v>9000.0</v>
+        <v>3000.0</v>
       </c>
       <c r="M8" t="inlineStr" s="0">
         <is>
@@ -390,60 +391,60 @@
     <row r="9">
       <c r="A9" t="inlineStr" s="0">
         <is>
-          <t>7. Broad Index &amp; Market Hedging</t>
+          <t>1. AI Chips &amp; Hardware</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="10">
         <is>
-          <t>QQQ</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="0">
         <is>
-          <t>Alpaca Live (#290523608)</t>
+          <t>Tradier Live (#6YB80974)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="10">
         <is>
-          <t>$700.00P / $675.00P</t>
+          <t>$605.00P / $600.00P</t>
         </is>
       </c>
       <c r="E9" s="0">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" s="6">
-        <v>742.03</v>
+        <v>633.91</v>
       </c>
       <c r="G9" t="inlineStr" s="7">
         <is>
-          <t>+$42.03 (+5.7%) OTM Buffer 🟢</t>
+          <t>+$28.91 (+4.6%) OTM Buffer 🟢</t>
         </is>
       </c>
       <c r="H9" s="6">
-        <v>368.0</v>
+        <v>513.0</v>
       </c>
       <c r="I9" s="6">
-        <v>168.0</v>
+        <v>413.0</v>
       </c>
       <c r="J9" s="7">
         <f>H9-I9</f>
-        <v>200.0</v>
+        <v>100.0</v>
       </c>
       <c r="K9" s="7">
         <f>J9*0.5</f>
-        <v>100.0</v>
+        <v>50.0</v>
       </c>
       <c r="L9" s="6">
-        <v>5000.0</v>
+        <v>500.0</v>
       </c>
       <c r="M9" t="inlineStr" s="0">
         <is>
-          <t>Oct 13, 2026 (T-3 DTE)</t>
+          <t>Oct 06, 2026 (T-3 DTE)</t>
         </is>
       </c>
       <c r="N9" t="inlineStr" s="0">
         <is>
-          <t>Oct 16, 2026</t>
+          <t>Oct 09, 2026</t>
         </is>
       </c>
       <c r="O9" t="inlineStr" s="7">
@@ -453,238 +454,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr" s="0">
-        <is>
-          <t>1. AI Chips &amp; Hardware</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr" s="10">
-        <is>
-          <t>TSM</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr" s="0">
-        <is>
-          <t>Alpaca Live (#290523608)</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr" s="10">
-        <is>
-          <t>$435.00P / $425.00P</t>
-        </is>
-      </c>
-      <c r="E10" s="0">
-        <v>3</v>
-      </c>
-      <c r="F10" s="6">
-        <v>459.2</v>
-      </c>
-      <c r="G10" t="inlineStr" s="7">
-        <is>
-          <t>+$24.20 (+5.3%) OTM Buffer 🟢</t>
-        </is>
-      </c>
-      <c r="H10" s="6">
-        <v>1485.0</v>
-      </c>
-      <c r="I10" s="6">
-        <v>930.0</v>
-      </c>
-      <c r="J10" s="7">
-        <f>H10-I10</f>
-        <v>555.0</v>
-      </c>
-      <c r="K10" s="7">
-        <f>J10*0.5</f>
-        <v>277.5</v>
-      </c>
-      <c r="L10" s="6">
-        <v>3000.0</v>
-      </c>
-      <c r="M10" t="inlineStr" s="0">
-        <is>
-          <t>Oct 13, 2026 (T-3 DTE)</t>
-        </is>
-      </c>
-      <c r="N10" t="inlineStr" s="0">
-        <is>
-          <t>Oct 16, 2026</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr" s="7">
-        <is>
-          <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr" s="0">
-        <is>
-          <t>3. Inflation Defense &amp; Hard Assets</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr" s="10">
-        <is>
-          <t>XLE</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr" s="0">
-        <is>
-          <t>Alpaca Live (#290523608)</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr" s="10">
-        <is>
-          <t>$60.00P / $58.00P</t>
-        </is>
-      </c>
-      <c r="E11" s="0">
-        <v>1</v>
-      </c>
-      <c r="F11" s="6">
-        <v>62.7</v>
-      </c>
-      <c r="G11" t="inlineStr" s="7">
-        <is>
-          <t>+$2.70 (+4.3%) OTM Buffer 🟢</t>
-        </is>
-      </c>
-      <c r="H11" s="6">
-        <v>68.0</v>
-      </c>
-      <c r="I11" s="6">
-        <v>32.0</v>
-      </c>
-      <c r="J11" s="7">
-        <f>H11-I11</f>
-        <v>36.0</v>
-      </c>
-      <c r="K11" s="7">
-        <f>J11*0.5</f>
-        <v>18.0</v>
-      </c>
-      <c r="L11" s="6">
-        <v>200.0</v>
-      </c>
-      <c r="M11" t="inlineStr" s="0">
-        <is>
-          <t>Oct 13, 2026 (T-3 DTE)</t>
-        </is>
-      </c>
-      <c r="N11" t="inlineStr" s="0">
-        <is>
-          <t>Oct 16, 2026</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr" s="7">
-        <is>
-          <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr" s="0">
-        <is>
-          <t>1. AI Chips &amp; Hardware</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr" s="10">
-        <is>
-          <t>TSM</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr" s="0">
-        <is>
-          <t>Tradier Live (#6YB80974)</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr" s="10">
-        <is>
-          <t>$425.00P / $420.00P</t>
-        </is>
-      </c>
-      <c r="E12" s="0">
-        <v>1</v>
-      </c>
-      <c r="F12" s="6">
-        <v>459.2</v>
-      </c>
-      <c r="G12" t="inlineStr" s="7">
-        <is>
-          <t>+$34.20 (+7.4%) OTM Buffer 🟢</t>
-        </is>
-      </c>
-      <c r="H12" s="6">
-        <v>897.0</v>
-      </c>
-      <c r="I12" s="6">
-        <v>747.0</v>
-      </c>
-      <c r="J12" s="7">
-        <f>H12-I12</f>
-        <v>150.0</v>
-      </c>
-      <c r="K12" s="7">
-        <f>J12*0.5</f>
-        <v>75.0</v>
-      </c>
-      <c r="L12" s="6">
-        <v>500.0</v>
-      </c>
-      <c r="M12" t="inlineStr" s="0">
-        <is>
-          <t>Oct 27, 2026 (T-3 DTE)</t>
-        </is>
-      </c>
-      <c r="N12" t="inlineStr" s="0">
-        <is>
-          <t>Oct 30, 2026</t>
-        </is>
-      </c>
-      <c r="O12" t="inlineStr" s="7">
-        <is>
-          <t>100% SAFE (Theta Burning on Schedule) 🟢</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr" s="5">
+      <c r="A10" t="inlineStr" s="5">
         <is>
           <t>PORTFOLIO TOTALS</t>
         </is>
       </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="13">
-        <f>SUM(E8:E12)</f>
-        <v>10</v>
-      </c>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="11">
-        <f>SUM(H8:H12)</f>
-        <v>3796.0</v>
-      </c>
-      <c r="I13" s="11">
-        <f>SUM(I8:I12)</f>
-        <v>1988.0</v>
-      </c>
-      <c r="J13" s="11">
-        <f>SUM(J8:J12)</f>
-        <v>1808.0</v>
-      </c>
-      <c r="K13" s="11">
-        <f>SUM(K8:K12)</f>
-        <v>904.0</v>
-      </c>
-      <c r="L13" s="11">
-        <f>SUM(L8:L12)</f>
-        <v>17700.0</v>
-      </c>
-      <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" t="inlineStr" s="5">
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="13">
+        <f>SUM(E8:E9)</f>
+        <v>4</v>
+      </c>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="11">
+        <f>SUM(H8:H9)</f>
+        <v>1683.0</v>
+      </c>
+      <c r="I10" s="11">
+        <f>SUM(I8:I9)</f>
+        <v>1124.0</v>
+      </c>
+      <c r="J10" s="11">
+        <f>SUM(J8:J9)</f>
+        <v>559.0</v>
+      </c>
+      <c r="K10" s="11">
+        <f>SUM(K8:K9)</f>
+        <v>279.5</v>
+      </c>
+      <c r="L10" s="11">
+        <f>SUM(L8:L9)</f>
+        <v>3500.0</v>
+      </c>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" t="inlineStr" s="5">
         <is>
           <t>100% DEFINED RISK PROTECTED ✅</t>
         </is>
@@ -970,7 +776,7 @@
       </c>
       <c r="Z5" t="inlineStr" s="0">
         <is>
-          <t>754fde1f-10f6-44f0-afc9-4d6b8f0ba882</t>
+          <t>ac0766e8-0d3b-4d3b-9826-b71e2ac092d0</t>
         </is>
       </c>
     </row>
@@ -1157,42 +963,44 @@
       </c>
       <c r="Q7" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R7" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>14:10:15</t>
         </is>
       </c>
       <c r="S7" s="6">
-        <v>0.0</v>
+        <v>0.32</v>
       </c>
       <c r="T7" s="6">
-        <v>0.0</v>
-      </c>
-      <c r="U7" s="6">
-        <v>0.00</v>
+        <v>32.0</v>
+      </c>
+      <c r="U7" s="7">
+        <f>O7-T7</f>
+        <v>4.0</v>
       </c>
       <c r="V7" s="8">
-        <v>0.0</v>
+        <f>IF(P7&gt;0,U7/P7,0)</f>
+        <v>0.02</v>
       </c>
       <c r="W7" s="0">
-        <v>0.0</v>
+        <v>258.8</v>
       </c>
       <c r="X7" t="inlineStr" s="0">
         <is>
-          <t>Active with broker (live position)</t>
+          <t>Take-profit close (verified fill)</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr" s="10">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED_HARVESTED</t>
         </is>
       </c>
       <c r="Z7" t="inlineStr" s="0">
         <is>
-          <t>e581bd48-ad5a-4ea2-b0b3-db33118a637b</t>
+          <t>cfbf1164-cbbb-4bd0-bc9c-27af3ce36483</t>
         </is>
       </c>
     </row>
@@ -1379,37 +1187,39 @@
       </c>
       <c r="Q9" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R9" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>13:35:15</t>
         </is>
       </c>
       <c r="S9" s="6">
-        <v>0.0</v>
+        <v>0.69</v>
       </c>
       <c r="T9" s="6">
-        <v>0.0</v>
-      </c>
-      <c r="U9" s="6">
-        <v>0.00</v>
+        <v>69.0</v>
+      </c>
+      <c r="U9" s="7">
+        <f>O9-T9</f>
+        <v>81.0</v>
       </c>
       <c r="V9" s="8">
-        <v>0.0</v>
+        <f>IF(P9&gt;0,U9/P9,0)</f>
+        <v>0.162</v>
       </c>
       <c r="W9" s="0">
-        <v>0.0</v>
+        <v>109.6</v>
       </c>
       <c r="X9" t="inlineStr" s="0">
         <is>
-          <t>Active with broker (live position)</t>
+          <t>Take-profit close (verified fill)</t>
         </is>
       </c>
       <c r="Y9" t="inlineStr" s="10">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED_HARVESTED</t>
         </is>
       </c>
       <c r="Z9" t="inlineStr" s="0">
@@ -1601,37 +1411,39 @@
       </c>
       <c r="Q11" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R11" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>14:55:11</t>
         </is>
       </c>
       <c r="S11" s="6">
-        <v>0.0</v>
+        <v>2.5</v>
       </c>
       <c r="T11" s="6">
-        <v>0.0</v>
-      </c>
-      <c r="U11" s="6">
-        <v>0.00</v>
+        <v>750.0</v>
+      </c>
+      <c r="U11" s="7">
+        <f>O11-T11</f>
+        <v>117.0</v>
       </c>
       <c r="V11" s="8">
-        <v>0.0</v>
+        <f>IF(P11&gt;0,U11/P11,0)</f>
+        <v>0.013</v>
       </c>
       <c r="W11" s="0">
-        <v>0.0</v>
+        <v>48.3</v>
       </c>
       <c r="X11" t="inlineStr" s="0">
         <is>
-          <t>Active with broker (live position)</t>
+          <t>Take-profit close (verified fill)</t>
         </is>
       </c>
       <c r="Y11" t="inlineStr" s="10">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED_HARVESTED</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr" s="0">
@@ -1738,7 +1550,7 @@
       </c>
       <c r="X12" t="inlineStr" s="0">
         <is>
-          <t>Take-profit close (verified fill) — rolled / re-entered 2x</t>
+          <t>Take-profit close (verified fill)</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr" s="10">
@@ -1748,7 +1560,7 @@
       </c>
       <c r="Z12" t="inlineStr" s="0">
         <is>
-          <t>18c2b2bd-a6f0-4943-a0c8-9f12613fbdde</t>
+          <t>903e39db-a575-4154-99fe-72bf672e2c5e</t>
         </is>
       </c>
     </row>
@@ -1823,42 +1635,44 @@
       </c>
       <c r="Q13" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R13" t="inlineStr" s="0">
         <is>
-          <t>-</t>
+          <t>13:30:19</t>
         </is>
       </c>
       <c r="S13" s="6">
-        <v>0.0</v>
+        <v>0.57</v>
       </c>
       <c r="T13" s="6">
-        <v>0.0</v>
-      </c>
-      <c r="U13" s="6">
-        <v>0.00</v>
+        <v>114.0</v>
+      </c>
+      <c r="U13" s="7">
+        <f>O13-T13</f>
+        <v>86.0</v>
       </c>
       <c r="V13" s="8">
-        <v>0.0</v>
+        <f>IF(P13&gt;0,U13/P13,0)</f>
+        <v>0.0172</v>
       </c>
       <c r="W13" s="0">
-        <v>0.0</v>
+        <v>46.3</v>
       </c>
       <c r="X13" t="inlineStr" s="0">
         <is>
-          <t>Active with broker (live position)</t>
+          <t>Take-profit close (verified fill)</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr" s="10">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED_HARVESTED</t>
         </is>
       </c>
       <c r="Z13" t="inlineStr" s="0">
         <is>
-          <t>a961797c-c700-495c-941e-0e0f66ab5a62</t>
+          <t>e268df2f-c894-47f6-8aea-9f1f91de236f</t>
         </is>
       </c>
     </row>
@@ -1933,97 +1747,721 @@
       </c>
       <c r="Q14" t="inlineStr" s="0">
         <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr" s="0">
+        <is>
+          <t>13:50:15</t>
+        </is>
+      </c>
+      <c r="S14" s="6">
+        <v>1.02</v>
+      </c>
+      <c r="T14" s="6">
+        <v>306.0</v>
+      </c>
+      <c r="U14" s="7">
+        <f>O14-T14</f>
+        <v>249.0</v>
+      </c>
+      <c r="V14" s="8">
+        <f>IF(P14&gt;0,U14/P14,0)</f>
+        <v>0.083</v>
+      </c>
+      <c r="W14" s="0">
+        <v>47.1</v>
+      </c>
+      <c r="X14" t="inlineStr" s="0">
+        <is>
+          <t>Take-profit close (verified fill)</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr" s="10">
+        <is>
+          <t>CLOSED_HARVESTED</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr" s="0">
+        <is>
+          <t>3b71756c-5bf9-4c7e-84b5-813ae535d313</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr" s="0">
+        <is>
+          <t>TRD-20261002-AMD-605/600</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr" s="0">
+        <is>
+          <t>Tradier Live (#6YB80974)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr" s="10">
+        <is>
+          <t>AMD</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr" s="0">
+        <is>
+          <t>1. AI Chips &amp; Hardware</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr" s="0">
+        <is>
+          <t>Bull Put Spread (605P/600P)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr" s="0">
+        <is>
+          <t>15:19:39</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr" s="0">
+        <is>
+          <t>AMD261009P00605000</t>
+        </is>
+      </c>
+      <c r="I15" s="6">
+        <v>605.0</v>
+      </c>
+      <c r="J15" t="inlineStr" s="0">
+        <is>
+          <t>AMD261009P00600000</t>
+        </is>
+      </c>
+      <c r="K15" s="6">
+        <v>600.0</v>
+      </c>
+      <c r="L15" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="M15" s="0">
+        <v>1</v>
+      </c>
+      <c r="N15" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="O15" s="6">
+        <v>100.0</v>
+      </c>
+      <c r="P15" s="6">
+        <v>500.0</v>
+      </c>
+      <c r="Q15" t="inlineStr" s="0">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="R14" t="inlineStr" s="0">
+      <c r="R15" t="inlineStr" s="0">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="S14" s="6">
+      <c r="S15" s="6">
         <v>0.0</v>
       </c>
-      <c r="T14" s="6">
+      <c r="T15" s="6">
         <v>0.0</v>
       </c>
-      <c r="U14" s="6">
+      <c r="U15" s="6">
         <v>0.00</v>
       </c>
-      <c r="V14" s="8">
+      <c r="V15" s="8">
         <v>0.0</v>
       </c>
-      <c r="W14" s="0">
+      <c r="W15" s="0">
         <v>0.0</v>
       </c>
-      <c r="X14" t="inlineStr" s="0">
+      <c r="X15" t="inlineStr" s="0">
         <is>
           <t>Active with broker (live position)</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr" s="10">
+      <c r="Y15" t="inlineStr" s="10">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="Z14" t="inlineStr" s="0">
-        <is>
-          <t>3b71756c-5bf9-4c7e-84b5-813ae535d313</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr" s="5">
+      <c r="Z15" t="inlineStr" s="0">
+        <is>
+          <t>149040437</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr" s="0">
+        <is>
+          <t>TRD-20261002-TSM-445/435</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (#290523608)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr" s="10">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr" s="0">
+        <is>
+          <t>1. AI Chips &amp; Hardware</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr" s="0">
+        <is>
+          <t>Bull Put Spread (445P/435P)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr" s="0">
+        <is>
+          <t>14:47:11</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr" s="0">
+        <is>
+          <t>TSM261016P00445000</t>
+        </is>
+      </c>
+      <c r="I16" s="6">
+        <v>445.0</v>
+      </c>
+      <c r="J16" t="inlineStr" s="0">
+        <is>
+          <t>TSM261016P00435000</t>
+        </is>
+      </c>
+      <c r="K16" s="6">
+        <v>435.0</v>
+      </c>
+      <c r="L16" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="M16" s="0">
+        <v>3</v>
+      </c>
+      <c r="N16" s="6">
+        <v>1.53</v>
+      </c>
+      <c r="O16" s="6">
+        <v>459.0</v>
+      </c>
+      <c r="P16" s="6">
+        <v>3000.0</v>
+      </c>
+      <c r="Q16" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr" s="0">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S16" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="T16" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="U16" s="6">
+        <v>0.00</v>
+      </c>
+      <c r="V16" s="8">
+        <v>0.0</v>
+      </c>
+      <c r="W16" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="X16" t="inlineStr" s="0">
+        <is>
+          <t>Active with broker (live position)</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr" s="10">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr" s="0">
+        <is>
+          <t>1e28c073-1f65-4de0-a3c2-972df8c2f7bc</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr" s="5">
         <is>
           <t>TOTALS / RECONCILED</t>
         </is>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5"/>
-      <c r="L15" s="5"/>
-      <c r="M15" s="13">
-        <f>SUM(M5:M14)</f>
-        <v>21</v>
-      </c>
-      <c r="N15" s="5"/>
-      <c r="O15" s="11">
-        <f>SUM(O5:O14)</f>
-        <v>2635.0</v>
-      </c>
-      <c r="P15" s="11">
-        <f>SUM(P5:P14)</f>
-        <v>26500.0</v>
-      </c>
-      <c r="Q15" s="5"/>
-      <c r="R15" s="5"/>
-      <c r="S15" s="5"/>
-      <c r="T15" s="11">
-        <f>SUM(T5:T14)</f>
-        <v>726.0</v>
-      </c>
-      <c r="U15" s="11">
-        <f>SUM(U5:U14)</f>
-        <v>101.0</v>
-      </c>
-      <c r="V15" s="5"/>
-      <c r="W15" s="5"/>
-      <c r="X15" s="5"/>
-      <c r="Y15" s="5"/>
-      <c r="Z15" s="5"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="13">
+        <f>SUM(M5:M16)</f>
+        <v>25</v>
+      </c>
+      <c r="N17" s="5"/>
+      <c r="O17" s="11">
+        <f>SUM(O5:O16)</f>
+        <v>3194.0</v>
+      </c>
+      <c r="P17" s="11">
+        <f>SUM(P5:P16)</f>
+        <v>30000.0</v>
+      </c>
+      <c r="Q17" s="5"/>
+      <c r="R17" s="5"/>
+      <c r="S17" s="5"/>
+      <c r="T17" s="11">
+        <f>SUM(T5:T16)</f>
+        <v>1997.0</v>
+      </c>
+      <c r="U17" s="11">
+        <f>SUM(U5:U16)</f>
+        <v>638.0</v>
+      </c>
+      <c r="V17" s="5"/>
+      <c r="W17" s="5"/>
+      <c r="X17" s="5"/>
+      <c r="Y17" s="5"/>
+      <c r="Z17" s="5"/>
     </row>
   </sheetData>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="16"/>
+    <col min="2" max="2" width="28"/>
+    <col min="3" max="3" width="16"/>
+    <col min="4" max="4" width="26"/>
+    <col min="5" max="5" width="24"/>
+    <col min="6" max="6" width="26"/>
+    <col min="7" max="7" width="26"/>
+    <col min="8" max="8" width="32"/>
+    <col min="9" max="9" width="24"/>
+    <col min="10" max="10" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t>SKONVAULT INBOUND CAPITAL DEPOSIT &amp; WISE FX REMITTANCE AUDIT TRAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="2">
+        <is>
+          <t>Cross-Border Capital Infusion Log — Reconciled with Bank Receipts, Wise Transfers, &amp; Clearing Brokers</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr" s="4">
+        <is>
+          <t>Transfer Date</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="4">
+        <is>
+          <t>Receiving Brokerage</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="4">
+        <is>
+          <t>Target Account</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="4">
+        <is>
+          <t>Platform / Account Type</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="4">
+        <is>
+          <t>Injected Principal (USD)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="4">
+        <is>
+          <t>THB Principal Debited (THB)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr" s="4">
+        <is>
+          <t>Effective FX Rate (THB/USD)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr" s="4">
+        <is>
+          <t>Remittance Rail</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr" s="4">
+        <is>
+          <t>Clearing Status</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr" s="4">
+        <is>
+          <t>Strategic Allocation Memo</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Securities LLC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="0">
+        <is>
+          <t>290523608</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (Margin)</t>
+        </is>
+      </c>
+      <c r="E5" s="6">
+        <v>10431.65</v>
+      </c>
+      <c r="F5" s="9">
+        <v>345000.0</v>
+      </c>
+      <c r="G5" s="0">
+        <v>33.0724</v>
+      </c>
+      <c r="H5" t="inlineStr" s="0">
+        <is>
+          <t>Wise ACH to BMO Harris (Alpaca)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr" s="10">
+        <is>
+          <t>SETTLED / CREDITED 🟢</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr" s="0">
+        <is>
+          <t>Trading Capital Batch 4 (Bought 60 SGOV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Securities LLC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="0">
+        <is>
+          <t>290523608</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (Margin)</t>
+        </is>
+      </c>
+      <c r="E6" s="6">
+        <v>10596.1</v>
+      </c>
+      <c r="F6" s="9">
+        <v>351000.0</v>
+      </c>
+      <c r="G6" s="0">
+        <v>33.1254</v>
+      </c>
+      <c r="H6" t="inlineStr" s="0">
+        <is>
+          <t>Wise ACH to BMO Harris (Alpaca)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr" s="10">
+        <is>
+          <t>SETTLED / CREDITED 🟢</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr" s="0">
+        <is>
+          <t>Trading Capital Batch 3 (Bought 194 SGOV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Securities LLC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="0">
+        <is>
+          <t>290523608</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (Margin)</t>
+        </is>
+      </c>
+      <c r="E7" s="6">
+        <v>4492.24</v>
+      </c>
+      <c r="F7" s="9">
+        <v>148944.27</v>
+      </c>
+      <c r="G7" s="0">
+        <v>33.1559</v>
+      </c>
+      <c r="H7" t="inlineStr" s="0">
+        <is>
+          <t>Wise ACH / Domestic Wire</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr" s="10">
+        <is>
+          <t>SETTLED / CLEARED 🟢</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr" s="0">
+        <is>
+          <t>Trading Capital Batch 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Securities LLC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="0">
+        <is>
+          <t>290523608</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Live (Margin)</t>
+        </is>
+      </c>
+      <c r="E8" s="6">
+        <v>4498.33</v>
+      </c>
+      <c r="F8" s="9">
+        <v>150000.0</v>
+      </c>
+      <c r="G8" s="0">
+        <v>33.3457</v>
+      </c>
+      <c r="H8" t="inlineStr" s="0">
+        <is>
+          <t>Wise ACH / Domestic Wire</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr" s="10">
+        <is>
+          <t>SETTLED / CLEARED 🟢</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr" s="0">
+        <is>
+          <t>Trading Capital Batch 1 (Bought 44 SGOV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="0">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="0">
+        <is>
+          <t>Tradier (Apex Clearing Inc.)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="0">
+        <is>
+          <t>6YB80974</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="0">
+        <is>
+          <t>Tradier Live (Margin L4)</t>
+        </is>
+      </c>
+      <c r="E9" s="6">
+        <v>2000.0</v>
+      </c>
+      <c r="F9" s="9">
+        <v>64879.26</v>
+      </c>
+      <c r="G9" s="0">
+        <v>32.4396</v>
+      </c>
+      <c r="H9" t="inlineStr" s="0">
+        <is>
+          <t>Wise Wire to Apex Clearing</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr" s="10">
+        <is>
+          <t>SETTLED / CLEARED 🟢</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr" s="0">
+        <is>
+          <t>POC Options Capital (Bought 19 SGOV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="0">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="0">
+        <is>
+          <t>Interactive Brokers LLC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="0">
+        <is>
+          <t>U25439978</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="0">
+        <is>
+          <t>IBKR Pro (Margin)</t>
+        </is>
+      </c>
+      <c r="E10" s="6">
+        <v>2200.0</v>
+      </c>
+      <c r="F10" s="9">
+        <v>71915.03</v>
+      </c>
+      <c r="G10" s="0">
+        <v>32.6887</v>
+      </c>
+      <c r="H10" t="inlineStr" s="0">
+        <is>
+          <t>Wise Wire to Citi NY (IBKR)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr" s="10">
+        <is>
+          <t>SETTLED / CLEARED 🟢</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr" s="0">
+        <is>
+          <t>IBKR Strategic Reserve Capital</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="5">
+        <is>
+          <t>CUMULATIVE CAPITAL INFLOW</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="5">
+        <is>
+          <t>6 TRANSFERS</t>
+        </is>
+      </c>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="11">
+        <f>SUM(E5:E10)</f>
+        <v>34218.32</v>
+      </c>
+      <c r="F11" s="12">
+        <f>SUM(F5:F10)</f>
+        <v>1131738.56</v>
+      </c>
+      <c r="G11" s="11">
+        <f>F11/E11</f>
+        <v>33.0741</v>
+      </c>
+      <c r="H11" t="inlineStr" s="5">
+        <is>
+          <t>100% WISE DIRECT</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr" s="5">
+        <is>
+          <t>ALL CLEARED 🟢</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr" s="5">
+        <is>
+          <t>FULLY CREDITED TO BROKERS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="20"/>
@@ -2163,7 +2601,7 @@
       </c>
       <c r="L5" t="inlineStr" s="0">
         <is>
-          <t>754fde1f-10f6-44f0-afc9-4d6b8f0ba882</t>
+          <t>ac0766e8-0d3b-4d3b-9826-b71e2ac092d0</t>
         </is>
       </c>
     </row>
@@ -2223,12 +2661,12 @@
     <row r="7">
       <c r="A7" t="inlineStr" s="0">
         <is>
-          <t>TAX-20260928-NVDA-220/215</t>
+          <t>TAX-20260921-XLE-60/58</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="0">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="0">
@@ -2243,174 +2681,439 @@
       </c>
       <c r="E7" t="inlineStr" s="10">
         <is>
-          <t>NVDA</t>
+          <t>XLE</t>
         </is>
       </c>
       <c r="F7" s="6">
-        <v>426.0</v>
+        <v>36.0</v>
       </c>
       <c r="G7" s="6">
-        <v>402.0</v>
+        <v>32.0</v>
       </c>
       <c r="H7" s="7">
         <f>F7-G7</f>
-        <v>24.0</v>
+        <v>4.0</v>
       </c>
       <c r="I7" s="6">
         <v>36.5</v>
       </c>
       <c r="J7" s="9">
         <f>IF(H7&gt;0,H7*I7,0)</f>
-        <v>876.0</v>
+        <v>146.0</v>
       </c>
       <c r="K7" s="9">
         <f>J7</f>
-        <v>876.0</v>
+        <v>146.0</v>
       </c>
       <c r="L7" t="inlineStr" s="0">
         <is>
-          <t>b62cee06-2bd9-43c4-a8ce-53385fad4b19</t>
+          <t>cfbf1164-cbbb-4bd0-bc9c-27af3ce36483</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr" s="0">
         <is>
-          <t>TAX-20260929-META-685/680</t>
+          <t>TAX-20260928-NVDA-220/215</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="0">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t>Tradier (Apex Clearing Corp)</t>
+          <t>Alpaca Securities LLC</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="0">
         <is>
-          <t>6YB80974</t>
+          <t>290523608</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="10">
         <is>
-          <t>META</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="F8" s="6">
-        <v>98.0</v>
+        <v>426.0</v>
       </c>
       <c r="G8" s="6">
-        <v>67.0</v>
+        <v>402.0</v>
       </c>
       <c r="H8" s="7">
         <f>F8-G8</f>
-        <v>31.0</v>
+        <v>24.0</v>
       </c>
       <c r="I8" s="6">
         <v>36.5</v>
       </c>
       <c r="J8" s="9">
         <f>IF(H8&gt;0,H8*I8,0)</f>
-        <v>1131.5</v>
+        <v>876.0</v>
       </c>
       <c r="K8" s="9">
         <f>J8</f>
-        <v>1131.5</v>
+        <v>876.0</v>
       </c>
       <c r="L8" t="inlineStr" s="0">
         <is>
-          <t>tradier_2026-09-29</t>
+          <t>b62cee06-2bd9-43c4-a8ce-53385fad4b19</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr" s="0">
         <is>
-          <t>TAX-20260930-QQQ-775/800</t>
+          <t>TAX-20260928-TSM-425/420</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="0">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="0">
         <is>
-          <t>Alpaca Securities LLC</t>
+          <t>Tradier (Apex Clearing Corp)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="0">
         <is>
-          <t>290523608</t>
+          <t>6YB80974</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="10">
         <is>
-          <t>QQQ</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="F9" s="6">
-        <v>284.0</v>
+        <v>150.0</v>
       </c>
       <c r="G9" s="6">
-        <v>178.0</v>
+        <v>69.0</v>
       </c>
       <c r="H9" s="7">
         <f>F9-G9</f>
-        <v>106.0</v>
+        <v>81.0</v>
       </c>
       <c r="I9" s="6">
         <v>36.5</v>
       </c>
       <c r="J9" s="9">
         <f>IF(H9&gt;0,H9*I9,0)</f>
-        <v>3869.0</v>
+        <v>2956.5</v>
       </c>
       <c r="K9" s="9">
         <f>J9</f>
+        <v>2956.5</v>
+      </c>
+      <c r="L9" t="inlineStr" s="0">
+        <is>
+          <t>tradier_2026-09-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="0">
+        <is>
+          <t>TAX-20260929-META-685/680</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="0">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="0">
+        <is>
+          <t>Tradier (Apex Clearing Corp)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="0">
+        <is>
+          <t>6YB80974</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="10">
+        <is>
+          <t>META</t>
+        </is>
+      </c>
+      <c r="F10" s="6">
+        <v>98.0</v>
+      </c>
+      <c r="G10" s="6">
+        <v>67.0</v>
+      </c>
+      <c r="H10" s="7">
+        <f>F10-G10</f>
+        <v>31.0</v>
+      </c>
+      <c r="I10" s="6">
+        <v>36.5</v>
+      </c>
+      <c r="J10" s="9">
+        <f>IF(H10&gt;0,H10*I10,0)</f>
+        <v>1131.5</v>
+      </c>
+      <c r="K10" s="9">
+        <f>J10</f>
+        <v>1131.5</v>
+      </c>
+      <c r="L10" t="inlineStr" s="0">
+        <is>
+          <t>tradier_2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="0">
+        <is>
+          <t>TAX-20260930-AVGO-335/305</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Securities LLC</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="0">
+        <is>
+          <t>290523608</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="10">
+        <is>
+          <t>AVGO</t>
+        </is>
+      </c>
+      <c r="F11" s="6">
+        <v>867.0</v>
+      </c>
+      <c r="G11" s="6">
+        <v>750.0</v>
+      </c>
+      <c r="H11" s="7">
+        <f>F11-G11</f>
+        <v>117.0</v>
+      </c>
+      <c r="I11" s="6">
+        <v>36.5</v>
+      </c>
+      <c r="J11" s="9">
+        <f>IF(H11&gt;0,H11*I11,0)</f>
+        <v>4270.5</v>
+      </c>
+      <c r="K11" s="9">
+        <f>J11</f>
+        <v>4270.5</v>
+      </c>
+      <c r="L11" t="inlineStr" s="0">
+        <is>
+          <t>9e306619-a4b3-4116-9ebf-df20c399e587</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="0">
+        <is>
+          <t>TAX-20260930-QQQ-775/800</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Securities LLC</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="0">
+        <is>
+          <t>290523608</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr" s="10">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="F12" s="6">
+        <v>284.0</v>
+      </c>
+      <c r="G12" s="6">
+        <v>178.0</v>
+      </c>
+      <c r="H12" s="7">
+        <f>F12-G12</f>
+        <v>106.0</v>
+      </c>
+      <c r="I12" s="6">
+        <v>36.5</v>
+      </c>
+      <c r="J12" s="9">
+        <f>IF(H12&gt;0,H12*I12,0)</f>
         <v>3869.0</v>
       </c>
-      <c r="L9" t="inlineStr" s="0">
-        <is>
-          <t>18c2b2bd-a6f0-4943-a0c8-9f12613fbdde</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr" s="5">
+      <c r="K12" s="9">
+        <f>J12</f>
+        <v>3869.0</v>
+      </c>
+      <c r="L12" t="inlineStr" s="0">
+        <is>
+          <t>903e39db-a575-4154-99fe-72bf672e2c5e</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr" s="0">
+        <is>
+          <t>TAX-20260930-QQQ-700/675</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Securities LLC</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="0">
+        <is>
+          <t>290523608</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="10">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="F13" s="6">
+        <v>200.0</v>
+      </c>
+      <c r="G13" s="6">
+        <v>114.0</v>
+      </c>
+      <c r="H13" s="7">
+        <f>F13-G13</f>
+        <v>86.0</v>
+      </c>
+      <c r="I13" s="6">
+        <v>36.5</v>
+      </c>
+      <c r="J13" s="9">
+        <f>IF(H13&gt;0,H13*I13,0)</f>
+        <v>3139.0</v>
+      </c>
+      <c r="K13" s="9">
+        <f>J13</f>
+        <v>3139.0</v>
+      </c>
+      <c r="L13" t="inlineStr" s="0">
+        <is>
+          <t>e268df2f-c894-47f6-8aea-9f1f91de236f</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr" s="0">
+        <is>
+          <t>TAX-20260930-TSM-435/425</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="0">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="0">
+        <is>
+          <t>Alpaca Securities LLC</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="0">
+        <is>
+          <t>290523608</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr" s="10">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="F14" s="6">
+        <v>555.0</v>
+      </c>
+      <c r="G14" s="6">
+        <v>306.0</v>
+      </c>
+      <c r="H14" s="7">
+        <f>F14-G14</f>
+        <v>249.0</v>
+      </c>
+      <c r="I14" s="6">
+        <v>36.5</v>
+      </c>
+      <c r="J14" s="9">
+        <f>IF(H14&gt;0,H14*I14,0)</f>
+        <v>9088.5</v>
+      </c>
+      <c r="K14" s="9">
+        <f>J14</f>
+        <v>9088.5</v>
+      </c>
+      <c r="L14" t="inlineStr" s="0">
+        <is>
+          <t>3b71756c-5bf9-4c7e-84b5-813ae535d313</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr" s="5">
         <is>
           <t>TOTAL CLOSED REVENUE</t>
         </is>
       </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="11">
-        <f>SUM(F5:F9)</f>
-        <v>827.0</v>
-      </c>
-      <c r="G10" s="11">
-        <f>SUM(G5:G9)</f>
-        <v>726.0</v>
-      </c>
-      <c r="H10" s="11">
-        <f>SUM(H5:H9)</f>
-        <v>101.0</v>
-      </c>
-      <c r="I10" s="5"/>
-      <c r="J10" s="12">
-        <f>SUM(J5:J9)</f>
-        <v>5876.5</v>
-      </c>
-      <c r="K10" s="12">
-        <f>SUM(K5:K9)</f>
-        <v>5876.5</v>
-      </c>
-      <c r="L10" t="inlineStr" s="5">
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="11">
+        <f>SUM(F5:F14)</f>
+        <v>2635.0</v>
+      </c>
+      <c r="G15" s="11">
+        <f>SUM(G5:G14)</f>
+        <v>1997.0</v>
+      </c>
+      <c r="H15" s="11">
+        <f>SUM(H5:H14)</f>
+        <v>638.0</v>
+      </c>
+      <c r="I15" s="5"/>
+      <c r="J15" s="12">
+        <f>SUM(J5:J14)</f>
+        <v>25477.0</v>
+      </c>
+      <c r="K15" s="12">
+        <f>SUM(K5:K14)</f>
+        <v>25477.0</v>
+      </c>
+      <c r="L15" t="inlineStr" s="5">
         <is>
           <t>AUDITED COMPLIANT ✅</t>
         </is>

</xml_diff>

<commit_message>
feat(pacing): formalize 70% capital utilization ceiling with merit-score multi-asset deployment and width-adaptive sizing
</commit_message>
<xml_diff>
--- a/SkonVault_Live_Transaction_Journal.xlsx
+++ b/SkonVault_Live_Transaction_Journal.xlsx
@@ -185,7 +185,7 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
         <is>
-          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-10-03 06:43 ICT</t>
+          <t>Executive Live Telemetry: 72h Weekend Theta Compounding &amp; Rollover Radar — As of 2026-10-03 22:27 ICT</t>
         </is>
       </c>
     </row>
@@ -223,10 +223,10 @@
     </row>
     <row r="5">
       <c r="A5" s="6">
-        <v>33271.32</v>
+        <v>33271.1</v>
       </c>
       <c r="C5" s="6">
-        <v>11427.61</v>
+        <v>11427.53</v>
       </c>
       <c r="E5" s="7">
         <f>J10</f>
@@ -356,10 +356,10 @@
         </is>
       </c>
       <c r="H8" s="6">
-        <v>1170.0</v>
+        <v>1183.5</v>
       </c>
       <c r="I8" s="6">
-        <v>711.0</v>
+        <v>724.5</v>
       </c>
       <c r="J8" s="7">
         <f>H8-I8</f>
@@ -470,11 +470,11 @@
       <c r="G10" s="5"/>
       <c r="H10" s="11">
         <f>SUM(H8:H9)</f>
-        <v>1683.0</v>
+        <v>1696.5</v>
       </c>
       <c r="I10" s="11">
         <f>SUM(I8:I9)</f>
-        <v>1124.0</v>
+        <v>1137.5</v>
       </c>
       <c r="J10" s="11">
         <f>SUM(J8:J9)</f>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="R9" t="inlineStr" s="0">
         <is>
-          <t>13:35:15</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="S9" s="6">
@@ -1210,7 +1210,7 @@
         <v>0.162</v>
       </c>
       <c r="W9" s="0">
-        <v>109.6</v>
+        <v>96.0</v>
       </c>
       <c r="X9" t="inlineStr" s="0">
         <is>
@@ -1821,7 +1821,7 @@
       </c>
       <c r="G15" t="inlineStr" s="0">
         <is>
-          <t>15:19:39</t>
+          <t>00:00:00</t>
         </is>
       </c>
       <c r="H15" t="inlineStr" s="0">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="Z15" t="inlineStr" s="0">
         <is>
-          <t>149040437</t>
+          <t>tradier_2026-10-02</t>
         </is>
       </c>
     </row>

</xml_diff>